<commit_message>
Fix Run 39 and Run 54, confirm geometry winners with full 30/30 valid data
Grand_Output_2.xlsx shows both previously-diverged wall-thickness cases
(Run 39: tp/dpo=0.05 @ Re=15K; Run 54: tp/dpo=0.15 @ Re=30K) now converge
cleanly via the transient-then-Steady fix. All 54 geometry runs are done.

Recomputed PEC with the complete dataset (6/6 valid in every group, no
more NA gaps): dpo/dti=0.25 and tp/dpo=0.10 both remain the winners —
the earlier tentative picks are now confirmed, not overturned.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DUewHsWD72fWTrA8cwVfXx
</commit_message>
<xml_diff>
--- a/Parameter_Run_Tracking_Table.xlsx
+++ b/Parameter_Run_Tracking_Table.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -60,6 +60,10 @@
       <name val="Times New Roman"/>
       <color rgb="FF000000"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="10">
@@ -181,7 +185,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -311,6 +315,36 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2487,9 +2521,9 @@
       <c r="E7" s="6" t="n">
         <v>0.25</v>
       </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>How large the promoter is relative to the tube bore. Screened in Stage 2 at the winning Pt = 200 mm, wall ratio = 0.05 fixed. Winner (tentative): 0.25 — pending re-run of its diverged 15K Re case.</t>
+      <c r="F7" s="54" t="inlineStr">
+        <is>
+          <t>How large the promoter is relative to the tube bore. Screened in Stage 2 at the winning Pt = 200 mm, wall ratio = 0.05 fixed. Winner CONFIRMED 2026-10-07: 0.25 — highest mean PEC, all 6/6 Re points valid (previously-diverged 15K case now fixed).</t>
         </is>
       </c>
     </row>
@@ -2513,9 +2547,9 @@
       <c r="E8" s="6" t="n">
         <v>0.15</v>
       </c>
-      <c r="F8" s="5" t="inlineStr">
-        <is>
-          <t>How thick the promoter's own wall is relative to its size. Screened in Stage 3 at Pt = 200 mm, dpo/dti = 0.25 (Stage 2 winner). The 0.05 level is reused from Stage 2 (same geometry) — 0.10 and 0.15 are new runs, now complete.</t>
+      <c r="F8" s="54" t="inlineStr">
+        <is>
+          <t>How thick the promoter's own wall is relative to its size. Screened in Stage 3 at Pt = 200 mm, dpo/dti = 0.25 (Stage 2 winner). Winner CONFIRMED 2026-10-07: 0.10 — highest mean PEC, all 6/6 Re points valid in every group (previously-diverged 20K and 30K cases now fixed).</t>
         </is>
       </c>
     </row>
@@ -3307,11 +3341,11 @@
           <t>UPDATE 2026-10-07: Al2O3-MWCNT and Ag-MgO are now data-complete too — see the two sections below. Same mirror-thesis equations as Hybrid Nanofluid #1 above (density/Cp mixing, Maxwell k_hnp, Brinkman viscosity); only the pure-substance inputs differ.</t>
         </is>
       </c>
-      <c r="B53" s="7" t="n"/>
-      <c r="C53" s="7" t="n"/>
-      <c r="D53" s="7" t="n"/>
-      <c r="E53" s="7" t="n"/>
-      <c r="F53" s="7" t="n"/>
+      <c r="B53" s="13" t="n"/>
+      <c r="C53" s="13" t="n"/>
+      <c r="D53" s="13" t="n"/>
+      <c r="E53" s="13" t="n"/>
+      <c r="F53" s="14" t="n"/>
     </row>
     <row r="55" ht="20" customHeight="1">
       <c r="A55" s="15" t="inlineStr">
@@ -3319,11 +3353,11 @@
           <t>Hybrid Nanofluid #2 — Al2O3-MWCNT/Syltherm-800 — FINAL, fully sourced (same equations as Hybrid Nanofluid #1)</t>
         </is>
       </c>
-      <c r="B55" s="15" t="n"/>
-      <c r="C55" s="15" t="n"/>
-      <c r="D55" s="15" t="n"/>
-      <c r="E55" s="15" t="n"/>
-      <c r="F55" s="15" t="n"/>
+      <c r="B55" s="13" t="n"/>
+      <c r="C55" s="13" t="n"/>
+      <c r="D55" s="13" t="n"/>
+      <c r="E55" s="13" t="n"/>
+      <c r="F55" s="14" t="n"/>
     </row>
     <row r="56" ht="60" customHeight="1">
       <c r="A56" s="7" t="inlineStr">
@@ -3331,11 +3365,11 @@
           <t>Deep web search 2026-10-06/07 across independent sources (not the mirror thesis, which cites no reference for these two). Al2O3 rho/Cp/k are essentially universal in nanofluid literature (matches mirror exactly). MWCNT rho/Cp cross-checked across 2+ independent sources. ONE OPEN FLAG: k_MWCNT=3000 W/m-K is the individual-tube / nanofluid-CFD-convention value used in virtually every published Al2O3-MWCNT hybrid paper — real bulk/bundled MWCNT measures far lower (~200 W/m-K in solid-state physics literature). Using 3000 matches the body of work this thesis is consistent with; flagged here so it is a documented choice, not a hidden assumption.</t>
         </is>
       </c>
-      <c r="B56" s="7" t="n"/>
-      <c r="C56" s="7" t="n"/>
-      <c r="D56" s="7" t="n"/>
-      <c r="E56" s="7" t="n"/>
-      <c r="F56" s="7" t="n"/>
+      <c r="B56" s="13" t="n"/>
+      <c r="C56" s="13" t="n"/>
+      <c r="D56" s="13" t="n"/>
+      <c r="E56" s="13" t="n"/>
+      <c r="F56" s="14" t="n"/>
     </row>
     <row r="58" ht="18" customHeight="1">
       <c r="A58" s="3" t="inlineStr">
@@ -3343,11 +3377,11 @@
           <t>Step 1 — pure-substance properties</t>
         </is>
       </c>
-      <c r="B58" s="3" t="n"/>
-      <c r="C58" s="3" t="n"/>
-      <c r="D58" s="3" t="n"/>
-      <c r="E58" s="3" t="n"/>
-      <c r="F58" s="3" t="n"/>
+      <c r="B58" s="13" t="n"/>
+      <c r="C58" s="13" t="n"/>
+      <c r="D58" s="13" t="n"/>
+      <c r="E58" s="13" t="n"/>
+      <c r="F58" s="14" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
@@ -3463,11 +3497,11 @@
           <t>Step 2 — worked example at phi=2%, 50:50 split, T_in=500K — ready to type into Fluent (equations: see Hybrid #1, Step 3 above)</t>
         </is>
       </c>
-      <c r="B64" s="3" t="n"/>
-      <c r="C64" s="3" t="n"/>
-      <c r="D64" s="3" t="n"/>
-      <c r="E64" s="3" t="n"/>
-      <c r="F64" s="3" t="n"/>
+      <c r="B64" s="13" t="n"/>
+      <c r="C64" s="13" t="n"/>
+      <c r="D64" s="13" t="n"/>
+      <c r="E64" s="13" t="n"/>
+      <c r="F64" s="14" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
@@ -3597,11 +3631,11 @@
           <t>GREEN LIGHT (with one flagged convention): all four properties sourced and pass the phi=0 sanity check. k_hnf and mu_hnf come out numerically identical to Fe2O3-GO's — this is a real model property (Maxwell saturates once particle k &gt;&gt; base-fluid k; Brinkman ignores particle identity entirely), not a calculation error.</t>
         </is>
       </c>
-      <c r="B72" s="23" t="n"/>
-      <c r="C72" s="23" t="n"/>
-      <c r="D72" s="23" t="n"/>
-      <c r="E72" s="23" t="n"/>
-      <c r="F72" s="23" t="n"/>
+      <c r="B72" s="13" t="n"/>
+      <c r="C72" s="13" t="n"/>
+      <c r="D72" s="13" t="n"/>
+      <c r="E72" s="13" t="n"/>
+      <c r="F72" s="14" t="n"/>
     </row>
     <row r="73" ht="30" customHeight="1">
       <c r="A73" s="7" t="inlineStr">
@@ -3609,11 +3643,11 @@
           <t>Fluent setup: copy syltherm800_oil, rename (e.g. "Al2O3MWCNT_phi2_5050"), switch the 4 properties to Constant, enter the values above. Do not edit the original.</t>
         </is>
       </c>
-      <c r="B73" s="7" t="n"/>
-      <c r="C73" s="7" t="n"/>
-      <c r="D73" s="7" t="n"/>
-      <c r="E73" s="7" t="n"/>
-      <c r="F73" s="7" t="n"/>
+      <c r="B73" s="13" t="n"/>
+      <c r="C73" s="13" t="n"/>
+      <c r="D73" s="13" t="n"/>
+      <c r="E73" s="13" t="n"/>
+      <c r="F73" s="14" t="n"/>
     </row>
     <row r="75" ht="20" customHeight="1">
       <c r="A75" s="15" t="inlineStr">
@@ -3621,11 +3655,11 @@
           <t>Hybrid Nanofluid #3 — Ag-MgO/Syltherm-800 — FINAL, fully sourced (same equations as Hybrid Nanofluid #1)</t>
         </is>
       </c>
-      <c r="B75" s="15" t="n"/>
-      <c r="C75" s="15" t="n"/>
-      <c r="D75" s="15" t="n"/>
-      <c r="E75" s="15" t="n"/>
-      <c r="F75" s="15" t="n"/>
+      <c r="B75" s="13" t="n"/>
+      <c r="C75" s="13" t="n"/>
+      <c r="D75" s="13" t="n"/>
+      <c r="E75" s="13" t="n"/>
+      <c r="F75" s="14" t="n"/>
     </row>
     <row r="76" ht="58" customHeight="1">
       <c r="A76" s="7" t="inlineStr">
@@ -3633,11 +3667,11 @@
           <t>Deep web search 2026-10-06/07. Ag rho/Cp/k are standard metal constants, fully settled, no disagreement anywhere. MgO rho=3580 kg/m3 is consistent everywhere (mineral/periclase density). ONE OPEN FLAG: MgO Cp/k used here (955 J/kg-K, 45 W/m-K) come from Ag-MgO-specific hybrid-nanofluid literature and sit close to general ceramic-handbook values; a second published convention also exists (879 J/kg-K, 30 W/m-K) from other Ag-MgO papers — a modest spread (&lt;10% Cp, 1.5x k), documented not hidden.</t>
         </is>
       </c>
-      <c r="B76" s="7" t="n"/>
-      <c r="C76" s="7" t="n"/>
-      <c r="D76" s="7" t="n"/>
-      <c r="E76" s="7" t="n"/>
-      <c r="F76" s="7" t="n"/>
+      <c r="B76" s="13" t="n"/>
+      <c r="C76" s="13" t="n"/>
+      <c r="D76" s="13" t="n"/>
+      <c r="E76" s="13" t="n"/>
+      <c r="F76" s="14" t="n"/>
     </row>
     <row r="78" ht="18" customHeight="1">
       <c r="A78" s="3" t="inlineStr">
@@ -3645,11 +3679,11 @@
           <t>Step 1 — pure-substance properties</t>
         </is>
       </c>
-      <c r="B78" s="3" t="n"/>
-      <c r="C78" s="3" t="n"/>
-      <c r="D78" s="3" t="n"/>
-      <c r="E78" s="3" t="n"/>
-      <c r="F78" s="3" t="n"/>
+      <c r="B78" s="13" t="n"/>
+      <c r="C78" s="13" t="n"/>
+      <c r="D78" s="13" t="n"/>
+      <c r="E78" s="13" t="n"/>
+      <c r="F78" s="14" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="4" t="inlineStr">
@@ -3765,11 +3799,11 @@
           <t>Step 2 — worked example at phi=2%, 50:50 split, T_in=500K — ready to type into Fluent (equations: see Hybrid #1, Step 3 above)</t>
         </is>
       </c>
-      <c r="B84" s="3" t="n"/>
-      <c r="C84" s="3" t="n"/>
-      <c r="D84" s="3" t="n"/>
-      <c r="E84" s="3" t="n"/>
-      <c r="F84" s="3" t="n"/>
+      <c r="B84" s="13" t="n"/>
+      <c r="C84" s="13" t="n"/>
+      <c r="D84" s="13" t="n"/>
+      <c r="E84" s="13" t="n"/>
+      <c r="F84" s="14" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="4" t="inlineStr">
@@ -3899,11 +3933,11 @@
           <t>GREEN LIGHT (with one flagged convention): all four properties sourced and pass the phi=0 sanity check. k_hnf and mu_hnf again come out numerically identical to the other two hybrids' — same reason: Maxwell saturation + Brinkman's particle-independence. Differences in simulated PEC across the three nanofluid types will come entirely from rho_hnf/Cp_hnf, not from k or viscosity.</t>
         </is>
       </c>
-      <c r="B92" s="23" t="n"/>
-      <c r="C92" s="23" t="n"/>
-      <c r="D92" s="23" t="n"/>
-      <c r="E92" s="23" t="n"/>
-      <c r="F92" s="23" t="n"/>
+      <c r="B92" s="13" t="n"/>
+      <c r="C92" s="13" t="n"/>
+      <c r="D92" s="13" t="n"/>
+      <c r="E92" s="13" t="n"/>
+      <c r="F92" s="14" t="n"/>
     </row>
     <row r="93" ht="30" customHeight="1">
       <c r="A93" s="7" t="inlineStr">
@@ -3911,11 +3945,11 @@
           <t>Fluent setup: copy syltherm800_oil, rename (e.g. "AgMgO_phi2_5050"), switch the 4 properties to Constant, enter the values above. Do not edit the original.</t>
         </is>
       </c>
-      <c r="B93" s="7" t="n"/>
-      <c r="C93" s="7" t="n"/>
-      <c r="D93" s="7" t="n"/>
-      <c r="E93" s="7" t="n"/>
-      <c r="F93" s="7" t="n"/>
+      <c r="B93" s="13" t="n"/>
+      <c r="C93" s="13" t="n"/>
+      <c r="D93" s="13" t="n"/>
+      <c r="E93" s="13" t="n"/>
+      <c r="F93" s="14" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="39">
@@ -3928,8 +3962,8 @@
     <mergeCell ref="A56:F56"/>
     <mergeCell ref="A21:F21"/>
     <mergeCell ref="E39:F39"/>
+    <mergeCell ref="A55:F55"/>
     <mergeCell ref="B38:D38"/>
-    <mergeCell ref="A55:F55"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="E35:F35"/>
     <mergeCell ref="B37:D37"/>
@@ -5926,14 +5960,14 @@
       <c r="H47" s="35" t="n">
         <v>15000</v>
       </c>
-      <c r="I47" s="36" t="inlineStr">
-        <is>
-          <t>DIVERGED</t>
-        </is>
-      </c>
-      <c r="J47" s="37" t="inlineStr">
-        <is>
-          <t>Still diverged — REMAINING, not yet re-run (see Grand Output sheet, case #15)</t>
+      <c r="I47" s="52" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J47" s="55" t="inlineStr">
+        <is>
+          <t>FIXED 2026-10-07 — transient-then-Steady re-run converged cleanly. See Grand Output v2 sheet, case #15.</t>
         </is>
       </c>
       <c r="K47" s="16" t="n"/>
@@ -6074,9 +6108,9 @@
       <c r="Q50" s="16" t="n"/>
     </row>
     <row r="51" ht="18" customHeight="1">
-      <c r="A51" s="10" t="inlineStr">
-        <is>
-          <t>Result: dpo/dti = 0.25 selected (tentative) — highest PEC at 4 of the 5 valid Re points; 15K Re run diverged, excluded, re-run still pending.</t>
+      <c r="A51" s="51" t="inlineStr">
+        <is>
+          <t>Result: dpo/dti = 0.25 CONFIRMED — highest mean PEC across all 6/6 valid Re points (no exclusions, re-run complete). See Grand Output v2 sheet.</t>
         </is>
       </c>
       <c r="B51" s="13" t="n"/>
@@ -6640,14 +6674,14 @@
       <c r="H65" s="35" t="n">
         <v>30000</v>
       </c>
-      <c r="I65" s="36" t="inlineStr">
-        <is>
-          <t>NOT RUN</t>
-        </is>
-      </c>
-      <c r="J65" s="37" t="inlineStr">
-        <is>
-          <t>REMAINING — no valid data yet, not yet re-run (see Grand Output sheet, case #30)</t>
+      <c r="I65" s="52" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J65" s="55" t="inlineStr">
+        <is>
+          <t>FIXED 2026-10-07 — transient-then-Steady re-run converged cleanly. See Grand Output v2 sheet, case #30.</t>
         </is>
       </c>
       <c r="K65" s="16" t="n"/>
@@ -6659,9 +6693,9 @@
       <c r="Q65" s="16" t="n"/>
     </row>
     <row r="67" ht="18" customHeight="1">
-      <c r="A67" s="3" t="inlineStr">
-        <is>
-          <t>Stage 4 — Hybrid Nanofluid Type Screening (Pt=200mm confirmed; dpo/dti=0.25 tentative; tp/dpo still TBD — 4 diverged Stage-3 reruns in progress)</t>
+      <c r="A67" s="27" t="inlineStr">
+        <is>
+          <t>Stage 4 — Hybrid Nanofluid Type Screening (Pt=200mm CONFIRMED; dpo/dti=0.25 CONFIRMED; tp/dpo=0.10 CONFIRMED — all Stage 1-3 geometry now locked in)</t>
         </is>
       </c>
       <c r="B67" s="13" t="n"/>
@@ -6722,14 +6756,14 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F69" s="21" t="inlineStr">
-        <is>
-          <t>0.25 (tentative)</t>
-        </is>
-      </c>
-      <c r="G69" s="21" t="inlineStr">
-        <is>
-          <t>TBD (reruns in progress)</t>
+      <c r="F69" s="52" t="inlineStr">
+        <is>
+          <t>0.25</t>
+        </is>
+      </c>
+      <c r="G69" s="52" t="inlineStr">
+        <is>
+          <t>0.10</t>
         </is>
       </c>
       <c r="H69" s="21" t="n">
@@ -6789,14 +6823,14 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F70" s="21" t="inlineStr">
-        <is>
-          <t>0.25 (tentative)</t>
-        </is>
-      </c>
-      <c r="G70" s="21" t="inlineStr">
-        <is>
-          <t>TBD (reruns in progress)</t>
+      <c r="F70" s="52" t="inlineStr">
+        <is>
+          <t>0.25</t>
+        </is>
+      </c>
+      <c r="G70" s="52" t="inlineStr">
+        <is>
+          <t>0.10</t>
         </is>
       </c>
       <c r="H70" s="21" t="n">
@@ -6856,14 +6890,14 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F71" s="21" t="inlineStr">
-        <is>
-          <t>0.25 (tentative)</t>
-        </is>
-      </c>
-      <c r="G71" s="21" t="inlineStr">
-        <is>
-          <t>TBD (reruns in progress)</t>
+      <c r="F71" s="52" t="inlineStr">
+        <is>
+          <t>0.25</t>
+        </is>
+      </c>
+      <c r="G71" s="52" t="inlineStr">
+        <is>
+          <t>0.10</t>
         </is>
       </c>
       <c r="H71" s="21" t="n">
@@ -6923,14 +6957,14 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F72" s="21" t="inlineStr">
-        <is>
-          <t>0.25 (tentative)</t>
-        </is>
-      </c>
-      <c r="G72" s="21" t="inlineStr">
-        <is>
-          <t>TBD (reruns in progress)</t>
+      <c r="F72" s="52" t="inlineStr">
+        <is>
+          <t>0.25</t>
+        </is>
+      </c>
+      <c r="G72" s="52" t="inlineStr">
+        <is>
+          <t>0.10</t>
         </is>
       </c>
       <c r="H72" s="21" t="n">
@@ -6990,14 +7024,14 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F73" s="21" t="inlineStr">
-        <is>
-          <t>0.25 (tentative)</t>
-        </is>
-      </c>
-      <c r="G73" s="21" t="inlineStr">
-        <is>
-          <t>TBD (reruns in progress)</t>
+      <c r="F73" s="52" t="inlineStr">
+        <is>
+          <t>0.25</t>
+        </is>
+      </c>
+      <c r="G73" s="52" t="inlineStr">
+        <is>
+          <t>0.10</t>
         </is>
       </c>
       <c r="H73" s="21" t="n">
@@ -7057,14 +7091,14 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F74" s="21" t="inlineStr">
-        <is>
-          <t>0.25 (tentative)</t>
-        </is>
-      </c>
-      <c r="G74" s="21" t="inlineStr">
-        <is>
-          <t>TBD (reruns in progress)</t>
+      <c r="F74" s="52" t="inlineStr">
+        <is>
+          <t>0.25</t>
+        </is>
+      </c>
+      <c r="G74" s="52" t="inlineStr">
+        <is>
+          <t>0.10</t>
         </is>
       </c>
       <c r="H74" s="21" t="n">
@@ -7124,14 +7158,14 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F75" s="24" t="inlineStr">
-        <is>
-          <t>0.25 (tentative)</t>
-        </is>
-      </c>
-      <c r="G75" s="24" t="inlineStr">
-        <is>
-          <t>TBD (reruns in progress)</t>
+      <c r="F75" s="53" t="inlineStr">
+        <is>
+          <t>0.25</t>
+        </is>
+      </c>
+      <c r="G75" s="53" t="inlineStr">
+        <is>
+          <t>0.10</t>
         </is>
       </c>
       <c r="H75" s="24" t="n">
@@ -7191,14 +7225,14 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F76" s="24" t="inlineStr">
-        <is>
-          <t>0.25 (tentative)</t>
-        </is>
-      </c>
-      <c r="G76" s="24" t="inlineStr">
-        <is>
-          <t>TBD (reruns in progress)</t>
+      <c r="F76" s="53" t="inlineStr">
+        <is>
+          <t>0.25</t>
+        </is>
+      </c>
+      <c r="G76" s="53" t="inlineStr">
+        <is>
+          <t>0.10</t>
         </is>
       </c>
       <c r="H76" s="24" t="n">
@@ -7258,14 +7292,14 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F77" s="24" t="inlineStr">
-        <is>
-          <t>0.25 (tentative)</t>
-        </is>
-      </c>
-      <c r="G77" s="24" t="inlineStr">
-        <is>
-          <t>TBD (reruns in progress)</t>
+      <c r="F77" s="53" t="inlineStr">
+        <is>
+          <t>0.25</t>
+        </is>
+      </c>
+      <c r="G77" s="53" t="inlineStr">
+        <is>
+          <t>0.10</t>
         </is>
       </c>
       <c r="H77" s="24" t="n">
@@ -7325,14 +7359,14 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F78" s="24" t="inlineStr">
-        <is>
-          <t>0.25 (tentative)</t>
-        </is>
-      </c>
-      <c r="G78" s="24" t="inlineStr">
-        <is>
-          <t>TBD (reruns in progress)</t>
+      <c r="F78" s="53" t="inlineStr">
+        <is>
+          <t>0.25</t>
+        </is>
+      </c>
+      <c r="G78" s="53" t="inlineStr">
+        <is>
+          <t>0.10</t>
         </is>
       </c>
       <c r="H78" s="24" t="n">
@@ -7392,14 +7426,14 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F79" s="24" t="inlineStr">
-        <is>
-          <t>0.25 (tentative)</t>
-        </is>
-      </c>
-      <c r="G79" s="24" t="inlineStr">
-        <is>
-          <t>TBD (reruns in progress)</t>
+      <c r="F79" s="53" t="inlineStr">
+        <is>
+          <t>0.25</t>
+        </is>
+      </c>
+      <c r="G79" s="53" t="inlineStr">
+        <is>
+          <t>0.10</t>
         </is>
       </c>
       <c r="H79" s="24" t="n">
@@ -7459,14 +7493,14 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F80" s="24" t="inlineStr">
-        <is>
-          <t>0.25 (tentative)</t>
-        </is>
-      </c>
-      <c r="G80" s="24" t="inlineStr">
-        <is>
-          <t>TBD (reruns in progress)</t>
+      <c r="F80" s="53" t="inlineStr">
+        <is>
+          <t>0.25</t>
+        </is>
+      </c>
+      <c r="G80" s="53" t="inlineStr">
+        <is>
+          <t>0.10</t>
         </is>
       </c>
       <c r="H80" s="24" t="n">
@@ -7526,14 +7560,14 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F81" s="24" t="inlineStr">
-        <is>
-          <t>0.25 (tentative)</t>
-        </is>
-      </c>
-      <c r="G81" s="24" t="inlineStr">
-        <is>
-          <t>TBD (reruns in progress)</t>
+      <c r="F81" s="53" t="inlineStr">
+        <is>
+          <t>0.25</t>
+        </is>
+      </c>
+      <c r="G81" s="53" t="inlineStr">
+        <is>
+          <t>0.10</t>
         </is>
       </c>
       <c r="H81" s="24" t="n">
@@ -7593,14 +7627,14 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F82" s="24" t="inlineStr">
-        <is>
-          <t>0.25 (tentative)</t>
-        </is>
-      </c>
-      <c r="G82" s="24" t="inlineStr">
-        <is>
-          <t>TBD (reruns in progress)</t>
+      <c r="F82" s="53" t="inlineStr">
+        <is>
+          <t>0.25</t>
+        </is>
+      </c>
+      <c r="G82" s="53" t="inlineStr">
+        <is>
+          <t>0.10</t>
         </is>
       </c>
       <c r="H82" s="24" t="n">
@@ -7660,14 +7694,14 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F83" s="24" t="inlineStr">
-        <is>
-          <t>0.25 (tentative)</t>
-        </is>
-      </c>
-      <c r="G83" s="24" t="inlineStr">
-        <is>
-          <t>TBD (reruns in progress)</t>
+      <c r="F83" s="53" t="inlineStr">
+        <is>
+          <t>0.25</t>
+        </is>
+      </c>
+      <c r="G83" s="53" t="inlineStr">
+        <is>
+          <t>0.10</t>
         </is>
       </c>
       <c r="H83" s="24" t="n">
@@ -7727,14 +7761,14 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F84" s="24" t="inlineStr">
-        <is>
-          <t>0.25 (tentative)</t>
-        </is>
-      </c>
-      <c r="G84" s="24" t="inlineStr">
-        <is>
-          <t>TBD (reruns in progress)</t>
+      <c r="F84" s="53" t="inlineStr">
+        <is>
+          <t>0.25</t>
+        </is>
+      </c>
+      <c r="G84" s="53" t="inlineStr">
+        <is>
+          <t>0.10</t>
         </is>
       </c>
       <c r="H84" s="24" t="n">
@@ -7794,14 +7828,14 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F85" s="24" t="inlineStr">
-        <is>
-          <t>0.25 (tentative)</t>
-        </is>
-      </c>
-      <c r="G85" s="24" t="inlineStr">
-        <is>
-          <t>TBD (reruns in progress)</t>
+      <c r="F85" s="53" t="inlineStr">
+        <is>
+          <t>0.25</t>
+        </is>
+      </c>
+      <c r="G85" s="53" t="inlineStr">
+        <is>
+          <t>0.10</t>
         </is>
       </c>
       <c r="H85" s="24" t="n">
@@ -7861,14 +7895,14 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F86" s="24" t="inlineStr">
-        <is>
-          <t>0.25 (tentative)</t>
-        </is>
-      </c>
-      <c r="G86" s="24" t="inlineStr">
-        <is>
-          <t>TBD (reruns in progress)</t>
+      <c r="F86" s="53" t="inlineStr">
+        <is>
+          <t>0.25</t>
+        </is>
+      </c>
+      <c r="G86" s="53" t="inlineStr">
+        <is>
+          <t>0.10</t>
         </is>
       </c>
       <c r="H86" s="24" t="n">
@@ -7966,9 +8000,9 @@
       <c r="J89" s="14" t="n"/>
     </row>
     <row r="90">
-      <c r="A90" s="7" t="inlineStr">
-        <is>
-          <t>Done: 52   |   Fixed 2026-10-04 (now Done): 2 (Run 47, Run 52)   |   Remaining (diverged / not run): 2 (Run 39, Run 54)</t>
+      <c r="A90" s="33" t="inlineStr">
+        <is>
+          <t>Done: 54  |  Fixed 2026-10-04: 2 (Run 47, Run 52)  |  Fixed 2026-10-07: 2 (Run 39, Run 54)  |  Remaining: 0 — all 54 geometry runs complete.</t>
         </is>
       </c>
       <c r="B90" s="13" t="n"/>
@@ -7998,9 +8032,9 @@
       <c r="J91" s="14" t="n"/>
     </row>
     <row r="92">
-      <c r="A92" s="7" t="inlineStr">
-        <is>
-          <t>Open items: (1) Run 39 — dpo/dti=0.25, tp/dpo=0.05 @ Re=15,000 — still diverged, re-run pending. (2) Run 54 — dpo/dti=0.25, tp/dpo=0.15 @ Re=30,000 — not yet re-run. Both needed before the wall-thickness PEC decision (Grand Output sheet) is final.</t>
+      <c r="A92" s="33" t="inlineStr">
+        <is>
+          <t>Open items: none — all 4 previously-diverged runs (Run 39, 47, 52, 54) are now fixed and confirmed. Geometry decision final: dpo/dti=0.25, tp/dpo=0.10.</t>
         </is>
       </c>
       <c r="B92" s="13" t="n"/>
@@ -8051,13 +8085,13 @@
     <col width="13" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="40" customWidth="1" min="11" max="11"/>
+    <col width="44" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
-    <row r="1" ht="20" customHeight="1">
+    <row r="1" ht="22" customHeight="1">
       <c r="A1" s="26" t="inlineStr">
         <is>
-          <t>Grand Output — All 30 Promoter-Size + Wall-Thickness Runs (d_po/d_ti=0.25 block shared between both comparisons)</t>
+          <t>Grand Output v2 — All 30 Promoter-Size + Wall-Thickness Runs — ALL CASES NOW VALID (2026-10-07, Run 39 &amp; Run 54 fixed)</t>
         </is>
       </c>
       <c r="B1" s="13" t="n"/>
@@ -8074,7 +8108,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="27" t="inlineStr">
         <is>
-          <t>Section 1 — Raw Fluent Output (all 30 cases)</t>
+          <t>Section 1 — Raw Fluent Output (all 30 cases, 30/30 valid)</t>
         </is>
       </c>
       <c r="B3" s="13" t="n"/>
@@ -8146,1088 +8180,1068 @@
       </c>
     </row>
     <row r="5" ht="15" customHeight="1">
-      <c r="A5" s="42" t="n">
+      <c r="A5" s="46" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="42" t="n">
+      <c r="B5" s="46" t="n">
         <v>0.15</v>
       </c>
-      <c r="C5" s="42" t="n">
+      <c r="C5" s="46" t="n">
         <v>0.05</v>
       </c>
-      <c r="D5" s="42" t="n">
+      <c r="D5" s="46" t="n">
         <v>5000</v>
       </c>
-      <c r="E5" s="42" t="n">
+      <c r="E5" s="46" t="n">
         <v>538.22</v>
       </c>
-      <c r="F5" s="42" t="n">
+      <c r="F5" s="46" t="n">
         <v>792.9</v>
       </c>
-      <c r="G5" s="42" t="n">
+      <c r="G5" s="46" t="n">
         <v>0.2077</v>
       </c>
-      <c r="H5" s="42" t="n">
+      <c r="H5" s="46" t="n">
         <v>0.03421</v>
       </c>
-      <c r="I5" s="42" t="n">
+      <c r="I5" s="46" t="n">
         <v>37764.9</v>
       </c>
-      <c r="J5" s="42" t="inlineStr">
+      <c r="J5" s="46" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="K5" s="43" t="inlineStr"/>
+      <c r="K5" s="47" t="inlineStr"/>
     </row>
     <row r="6" ht="15" customHeight="1">
-      <c r="A6" s="42" t="n">
+      <c r="A6" s="46" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="42" t="n">
+      <c r="B6" s="46" t="n">
         <v>0.15</v>
       </c>
-      <c r="C6" s="42" t="n">
+      <c r="C6" s="46" t="n">
         <v>0.05</v>
       </c>
-      <c r="D6" s="42" t="n">
+      <c r="D6" s="46" t="n">
         <v>10000</v>
       </c>
-      <c r="E6" s="42" t="n">
+      <c r="E6" s="46" t="n">
         <v>519.16</v>
       </c>
-      <c r="F6" s="42" t="n">
+      <c r="F6" s="46" t="n">
         <v>682.76</v>
       </c>
-      <c r="G6" s="42" t="n">
+      <c r="G6" s="46" t="n">
         <v>0.4154</v>
       </c>
-      <c r="H6" s="42" t="n">
+      <c r="H6" s="46" t="n">
         <v>0.10793</v>
       </c>
-      <c r="I6" s="42" t="n">
+      <c r="I6" s="46" t="n">
         <v>37764.9</v>
       </c>
-      <c r="J6" s="42" t="inlineStr">
+      <c r="J6" s="46" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="K6" s="43" t="inlineStr"/>
+      <c r="K6" s="47" t="inlineStr"/>
     </row>
     <row r="7" ht="15" customHeight="1">
-      <c r="A7" s="42" t="n">
+      <c r="A7" s="46" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="42" t="n">
+      <c r="B7" s="46" t="n">
         <v>0.15</v>
       </c>
-      <c r="C7" s="42" t="n">
+      <c r="C7" s="46" t="n">
         <v>0.05</v>
       </c>
-      <c r="D7" s="42" t="n">
+      <c r="D7" s="46" t="n">
         <v>15000</v>
       </c>
-      <c r="E7" s="42" t="n">
+      <c r="E7" s="46" t="n">
         <v>512.79</v>
       </c>
-      <c r="F7" s="42" t="n">
+      <c r="F7" s="46" t="n">
         <v>633.13</v>
       </c>
-      <c r="G7" s="42" t="n">
+      <c r="G7" s="46" t="n">
         <v>0.6231</v>
       </c>
-      <c r="H7" s="42" t="n">
+      <c r="H7" s="46" t="n">
         <v>0.21607</v>
       </c>
-      <c r="I7" s="42" t="n">
+      <c r="I7" s="46" t="n">
         <v>37764.9</v>
       </c>
-      <c r="J7" s="42" t="inlineStr">
+      <c r="J7" s="46" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="K7" s="43" t="inlineStr"/>
+      <c r="K7" s="47" t="inlineStr"/>
     </row>
     <row r="8" ht="15" customHeight="1">
-      <c r="A8" s="42" t="n">
+      <c r="A8" s="46" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="42" t="n">
+      <c r="B8" s="46" t="n">
         <v>0.15</v>
       </c>
-      <c r="C8" s="42" t="n">
+      <c r="C8" s="46" t="n">
         <v>0.05</v>
       </c>
-      <c r="D8" s="42" t="n">
+      <c r="D8" s="46" t="n">
         <v>20000</v>
       </c>
-      <c r="E8" s="42" t="n">
+      <c r="E8" s="46" t="n">
         <v>509.59</v>
       </c>
-      <c r="F8" s="42" t="n">
+      <c r="F8" s="46" t="n">
         <v>606.1799999999999</v>
       </c>
-      <c r="G8" s="42" t="n">
+      <c r="G8" s="46" t="n">
         <v>0.8308</v>
       </c>
-      <c r="H8" s="42" t="n">
+      <c r="H8" s="46" t="n">
         <v>0.35269</v>
       </c>
-      <c r="I8" s="42" t="n">
+      <c r="I8" s="46" t="n">
         <v>37764.9</v>
       </c>
-      <c r="J8" s="42" t="inlineStr">
+      <c r="J8" s="46" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="K8" s="43" t="inlineStr"/>
+      <c r="K8" s="47" t="inlineStr"/>
     </row>
     <row r="9" ht="15" customHeight="1">
-      <c r="A9" s="42" t="n">
+      <c r="A9" s="46" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="42" t="n">
+      <c r="B9" s="46" t="n">
         <v>0.15</v>
       </c>
-      <c r="C9" s="42" t="n">
+      <c r="C9" s="46" t="n">
         <v>0.05</v>
       </c>
-      <c r="D9" s="42" t="n">
+      <c r="D9" s="46" t="n">
         <v>25000</v>
       </c>
-      <c r="E9" s="42" t="n">
+      <c r="E9" s="46" t="n">
         <v>507.68</v>
       </c>
-      <c r="F9" s="42" t="n">
+      <c r="F9" s="46" t="n">
         <v>589.62</v>
       </c>
-      <c r="G9" s="42" t="n">
+      <c r="G9" s="46" t="n">
         <v>1.0384</v>
       </c>
-      <c r="H9" s="42" t="n">
+      <c r="H9" s="46" t="n">
         <v>0.51334</v>
       </c>
-      <c r="I9" s="42" t="n">
+      <c r="I9" s="46" t="n">
         <v>37764.9</v>
       </c>
-      <c r="J9" s="42" t="inlineStr">
+      <c r="J9" s="46" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="K9" s="43" t="inlineStr"/>
+      <c r="K9" s="47" t="inlineStr"/>
     </row>
     <row r="10" ht="15" customHeight="1">
-      <c r="A10" s="42" t="n">
+      <c r="A10" s="46" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="42" t="n">
+      <c r="B10" s="46" t="n">
         <v>0.15</v>
       </c>
-      <c r="C10" s="42" t="n">
+      <c r="C10" s="46" t="n">
         <v>0.05</v>
       </c>
-      <c r="D10" s="42" t="n">
+      <c r="D10" s="46" t="n">
         <v>30000</v>
       </c>
-      <c r="E10" s="42" t="n">
+      <c r="E10" s="46" t="n">
         <v>506.4</v>
       </c>
-      <c r="F10" s="42" t="n">
+      <c r="F10" s="46" t="n">
         <v>578.3</v>
       </c>
-      <c r="G10" s="42" t="n">
+      <c r="G10" s="46" t="n">
         <v>1.2461</v>
       </c>
-      <c r="H10" s="42" t="n">
+      <c r="H10" s="46" t="n">
         <v>0.69404</v>
       </c>
-      <c r="I10" s="42" t="n">
+      <c r="I10" s="46" t="n">
         <v>37764.9</v>
       </c>
-      <c r="J10" s="42" t="inlineStr">
+      <c r="J10" s="46" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="K10" s="43" t="inlineStr"/>
+      <c r="K10" s="47" t="inlineStr"/>
     </row>
     <row r="11" ht="15" customHeight="1">
-      <c r="A11" s="42" t="n">
+      <c r="A11" s="46" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="42" t="n">
+      <c r="B11" s="46" t="n">
         <v>0.2</v>
       </c>
-      <c r="C11" s="42" t="n">
+      <c r="C11" s="46" t="n">
         <v>0.05</v>
       </c>
-      <c r="D11" s="42" t="n">
+      <c r="D11" s="46" t="n">
         <v>5000</v>
       </c>
-      <c r="E11" s="42" t="n">
+      <c r="E11" s="46" t="n">
         <v>538.4</v>
       </c>
-      <c r="F11" s="42" t="n">
+      <c r="F11" s="46" t="n">
         <v>782.0599999999999</v>
       </c>
-      <c r="G11" s="42" t="n">
+      <c r="G11" s="46" t="n">
         <v>0.2068</v>
       </c>
-      <c r="H11" s="42" t="n">
+      <c r="H11" s="46" t="n">
         <v>0.03562</v>
       </c>
-      <c r="I11" s="42" t="n">
+      <c r="I11" s="46" t="n">
         <v>37764.9</v>
       </c>
-      <c r="J11" s="42" t="inlineStr">
+      <c r="J11" s="46" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="K11" s="43" t="inlineStr"/>
+      <c r="K11" s="47" t="inlineStr"/>
     </row>
     <row r="12" ht="15" customHeight="1">
-      <c r="A12" s="42" t="n">
+      <c r="A12" s="46" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="42" t="n">
+      <c r="B12" s="46" t="n">
         <v>0.2</v>
       </c>
-      <c r="C12" s="42" t="n">
+      <c r="C12" s="46" t="n">
         <v>0.05</v>
       </c>
-      <c r="D12" s="42" t="n">
+      <c r="D12" s="46" t="n">
         <v>10000</v>
       </c>
-      <c r="E12" s="42" t="n">
+      <c r="E12" s="46" t="n">
         <v>519.25</v>
       </c>
-      <c r="F12" s="42" t="n">
+      <c r="F12" s="46" t="n">
         <v>678.0599999999999</v>
       </c>
-      <c r="G12" s="42" t="n">
+      <c r="G12" s="46" t="n">
         <v>0.4136</v>
       </c>
-      <c r="H12" s="42" t="n">
+      <c r="H12" s="46" t="n">
         <v>0.11198</v>
       </c>
-      <c r="I12" s="42" t="n">
+      <c r="I12" s="46" t="n">
         <v>37764.9</v>
       </c>
-      <c r="J12" s="42" t="inlineStr">
+      <c r="J12" s="46" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="K12" s="43" t="inlineStr"/>
+      <c r="K12" s="47" t="inlineStr"/>
     </row>
     <row r="13" ht="15" customHeight="1">
-      <c r="A13" s="42" t="n">
+      <c r="A13" s="46" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="42" t="n">
+      <c r="B13" s="46" t="n">
         <v>0.2</v>
       </c>
-      <c r="C13" s="42" t="n">
+      <c r="C13" s="46" t="n">
         <v>0.05</v>
       </c>
-      <c r="D13" s="42" t="n">
+      <c r="D13" s="46" t="n">
         <v>15000</v>
       </c>
-      <c r="E13" s="42" t="n">
+      <c r="E13" s="46" t="n">
         <v>512.84</v>
       </c>
-      <c r="F13" s="42" t="n">
+      <c r="F13" s="46" t="n">
         <v>630.3</v>
       </c>
-      <c r="G13" s="42" t="n">
+      <c r="G13" s="46" t="n">
         <v>0.6204</v>
       </c>
-      <c r="H13" s="42" t="n">
+      <c r="H13" s="46" t="n">
         <v>0.22359</v>
       </c>
-      <c r="I13" s="42" t="n">
+      <c r="I13" s="46" t="n">
         <v>37764.9</v>
       </c>
-      <c r="J13" s="42" t="inlineStr">
+      <c r="J13" s="46" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="K13" s="43" t="inlineStr"/>
+      <c r="K13" s="47" t="inlineStr"/>
     </row>
     <row r="14" ht="15" customHeight="1">
-      <c r="A14" s="42" t="n">
+      <c r="A14" s="46" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="42" t="n">
+      <c r="B14" s="46" t="n">
         <v>0.2</v>
       </c>
-      <c r="C14" s="42" t="n">
+      <c r="C14" s="46" t="n">
         <v>0.05</v>
       </c>
-      <c r="D14" s="42" t="n">
+      <c r="D14" s="46" t="n">
         <v>20000</v>
       </c>
-      <c r="E14" s="42" t="n">
+      <c r="E14" s="46" t="n">
         <v>509.64</v>
       </c>
-      <c r="F14" s="42" t="n">
+      <c r="F14" s="46" t="n">
         <v>604.1</v>
       </c>
-      <c r="G14" s="42" t="n">
+      <c r="G14" s="46" t="n">
         <v>0.8272</v>
       </c>
-      <c r="H14" s="42" t="n">
+      <c r="H14" s="46" t="n">
         <v>0.36497</v>
       </c>
-      <c r="I14" s="42" t="n">
+      <c r="I14" s="46" t="n">
         <v>37764.9</v>
       </c>
-      <c r="J14" s="42" t="inlineStr">
+      <c r="J14" s="46" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="K14" s="43" t="inlineStr"/>
+      <c r="K14" s="47" t="inlineStr"/>
     </row>
     <row r="15" ht="15" customHeight="1">
-      <c r="A15" s="42" t="n">
+      <c r="A15" s="46" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="42" t="n">
+      <c r="B15" s="46" t="n">
         <v>0.2</v>
       </c>
-      <c r="C15" s="42" t="n">
+      <c r="C15" s="46" t="n">
         <v>0.05</v>
       </c>
-      <c r="D15" s="42" t="n">
+      <c r="D15" s="46" t="n">
         <v>25000</v>
       </c>
-      <c r="E15" s="42" t="n">
+      <c r="E15" s="46" t="n">
         <v>507.71</v>
       </c>
-      <c r="F15" s="42" t="n">
+      <c r="F15" s="46" t="n">
         <v>587.92</v>
       </c>
-      <c r="G15" s="42" t="n">
+      <c r="G15" s="46" t="n">
         <v>1.034</v>
       </c>
-      <c r="H15" s="42" t="n">
+      <c r="H15" s="46" t="n">
         <v>0.53154</v>
       </c>
-      <c r="I15" s="42" t="n">
+      <c r="I15" s="46" t="n">
         <v>37764.9</v>
       </c>
-      <c r="J15" s="42" t="inlineStr">
+      <c r="J15" s="46" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="K15" s="43" t="inlineStr"/>
+      <c r="K15" s="47" t="inlineStr"/>
     </row>
     <row r="16" ht="15" customHeight="1">
-      <c r="A16" s="42" t="n">
+      <c r="A16" s="46" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="42" t="n">
+      <c r="B16" s="46" t="n">
         <v>0.2</v>
       </c>
-      <c r="C16" s="42" t="n">
+      <c r="C16" s="46" t="n">
         <v>0.05</v>
       </c>
-      <c r="D16" s="42" t="n">
+      <c r="D16" s="46" t="n">
         <v>30000</v>
       </c>
-      <c r="E16" s="42" t="n">
+      <c r="E16" s="46" t="n">
         <v>506.43</v>
       </c>
-      <c r="F16" s="42" t="n">
+      <c r="F16" s="46" t="n">
         <v>576.8099999999999</v>
       </c>
-      <c r="G16" s="42" t="n">
+      <c r="G16" s="46" t="n">
         <v>1.2408</v>
       </c>
-      <c r="H16" s="42" t="n">
+      <c r="H16" s="46" t="n">
         <v>0.71924</v>
       </c>
-      <c r="I16" s="42" t="n">
+      <c r="I16" s="46" t="n">
         <v>37764.9</v>
       </c>
-      <c r="J16" s="42" t="inlineStr">
+      <c r="J16" s="46" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="K16" s="43" t="inlineStr"/>
+      <c r="K16" s="47" t="inlineStr"/>
     </row>
     <row r="17" ht="15" customHeight="1">
-      <c r="A17" s="42" t="n">
+      <c r="A17" s="46" t="n">
         <v>13</v>
       </c>
-      <c r="B17" s="42" t="n">
+      <c r="B17" s="46" t="n">
         <v>0.25</v>
       </c>
-      <c r="C17" s="42" t="n">
+      <c r="C17" s="46" t="n">
         <v>0.05</v>
       </c>
-      <c r="D17" s="42" t="n">
+      <c r="D17" s="46" t="n">
         <v>5000</v>
       </c>
-      <c r="E17" s="42" t="n">
+      <c r="E17" s="46" t="n">
         <v>538.64</v>
       </c>
-      <c r="F17" s="42" t="n">
+      <c r="F17" s="46" t="n">
         <v>771.3</v>
       </c>
-      <c r="G17" s="42" t="n">
+      <c r="G17" s="46" t="n">
         <v>0.2057</v>
       </c>
-      <c r="H17" s="42" t="n">
+      <c r="H17" s="46" t="n">
         <v>0.03751</v>
       </c>
-      <c r="I17" s="42" t="n">
+      <c r="I17" s="46" t="n">
         <v>37764.9</v>
       </c>
-      <c r="J17" s="42" t="inlineStr">
+      <c r="J17" s="46" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="K17" s="43" t="inlineStr"/>
+      <c r="K17" s="47" t="inlineStr"/>
     </row>
     <row r="18" ht="15" customHeight="1">
-      <c r="A18" s="42" t="n">
+      <c r="A18" s="46" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="42" t="n">
+      <c r="B18" s="46" t="n">
         <v>0.25</v>
       </c>
-      <c r="C18" s="42" t="n">
+      <c r="C18" s="46" t="n">
         <v>0.05</v>
       </c>
-      <c r="D18" s="42" t="n">
+      <c r="D18" s="46" t="n">
         <v>10000</v>
       </c>
-      <c r="E18" s="42" t="n">
+      <c r="E18" s="46" t="n">
         <v>511.72</v>
       </c>
-      <c r="F18" s="42" t="n">
+      <c r="F18" s="46" t="n">
         <v>665.01</v>
       </c>
-      <c r="G18" s="42" t="n">
+      <c r="G18" s="46" t="n">
         <v>0.4113</v>
       </c>
-      <c r="H18" s="42" t="n">
+      <c r="H18" s="46" t="n">
         <v>0.13988</v>
       </c>
-      <c r="I18" s="42" t="n">
+      <c r="I18" s="46" t="n">
         <v>37764.9</v>
       </c>
-      <c r="J18" s="42" t="inlineStr">
+      <c r="J18" s="46" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="K18" s="43" t="inlineStr"/>
+      <c r="K18" s="47" t="inlineStr"/>
     </row>
     <row r="19" ht="15" customHeight="1">
-      <c r="A19" s="44" t="n">
+      <c r="A19" s="46" t="n">
         <v>15</v>
       </c>
-      <c r="B19" s="44" t="n">
+      <c r="B19" s="46" t="n">
         <v>0.25</v>
       </c>
-      <c r="C19" s="44" t="n">
+      <c r="C19" s="46" t="n">
         <v>0.05</v>
       </c>
-      <c r="D19" s="44" t="n">
+      <c r="D19" s="46" t="n">
         <v>15000</v>
       </c>
-      <c r="E19" s="44" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F19" s="44" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G19" s="44" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H19" s="44" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I19" s="44" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J19" s="44" t="inlineStr">
-        <is>
-          <t>DIVERGED</t>
-        </is>
-      </c>
-      <c r="K19" s="45" t="inlineStr">
-        <is>
-          <t>Still bad — remaining, not yet re-run</t>
+      <c r="E19" s="46" t="n">
+        <v>512.91</v>
+      </c>
+      <c r="F19" s="46" t="n">
+        <v>627.12</v>
+      </c>
+      <c r="G19" s="46" t="n">
+        <v>0.617</v>
+      </c>
+      <c r="H19" s="46" t="n">
+        <v>0.23329</v>
+      </c>
+      <c r="I19" s="46" t="n">
+        <v>37764.9</v>
+      </c>
+      <c r="J19" s="48" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="K19" s="49" t="inlineStr">
+        <is>
+          <t>Run 39 — re-run 2026-10-07 (transient-then-Steady fix); now converged cleanly</t>
         </is>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1">
-      <c r="A20" s="42" t="n">
+      <c r="A20" s="46" t="n">
         <v>16</v>
       </c>
-      <c r="B20" s="42" t="n">
+      <c r="B20" s="46" t="n">
         <v>0.25</v>
       </c>
-      <c r="C20" s="42" t="n">
+      <c r="C20" s="46" t="n">
         <v>0.05</v>
       </c>
-      <c r="D20" s="42" t="n">
+      <c r="D20" s="46" t="n">
         <v>20000</v>
       </c>
-      <c r="E20" s="42" t="n">
+      <c r="E20" s="46" t="n">
         <v>509.01</v>
       </c>
-      <c r="F20" s="42" t="n">
+      <c r="F20" s="46" t="n">
         <v>599.42</v>
       </c>
-      <c r="G20" s="42" t="n">
+      <c r="G20" s="46" t="n">
         <v>0.8227</v>
       </c>
-      <c r="H20" s="42" t="n">
+      <c r="H20" s="46" t="n">
         <v>0.42489</v>
       </c>
-      <c r="I20" s="42" t="n">
+      <c r="I20" s="46" t="n">
         <v>37764.5</v>
       </c>
-      <c r="J20" s="42" t="inlineStr">
+      <c r="J20" s="46" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="K20" s="43" t="inlineStr"/>
+      <c r="K20" s="47" t="inlineStr"/>
     </row>
     <row r="21" ht="15" customHeight="1">
-      <c r="A21" s="42" t="n">
+      <c r="A21" s="46" t="n">
         <v>17</v>
       </c>
-      <c r="B21" s="42" t="n">
+      <c r="B21" s="46" t="n">
         <v>0.25</v>
       </c>
-      <c r="C21" s="42" t="n">
+      <c r="C21" s="46" t="n">
         <v>0.05</v>
       </c>
-      <c r="D21" s="42" t="n">
+      <c r="D21" s="46" t="n">
         <v>25000</v>
       </c>
-      <c r="E21" s="42" t="n">
+      <c r="E21" s="46" t="n">
         <v>507.69</v>
       </c>
-      <c r="F21" s="42" t="n">
+      <c r="F21" s="46" t="n">
         <v>584.53</v>
       </c>
-      <c r="G21" s="42" t="n">
+      <c r="G21" s="46" t="n">
         <v>1.0283</v>
       </c>
-      <c r="H21" s="42" t="n">
+      <c r="H21" s="46" t="n">
         <v>0.59145</v>
       </c>
-      <c r="I21" s="42" t="n">
+      <c r="I21" s="46" t="n">
         <v>37765</v>
       </c>
-      <c r="J21" s="42" t="inlineStr">
+      <c r="J21" s="46" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="K21" s="43" t="inlineStr"/>
+      <c r="K21" s="47" t="inlineStr"/>
     </row>
     <row r="22" ht="15" customHeight="1">
-      <c r="A22" s="42" t="n">
+      <c r="A22" s="46" t="n">
         <v>18</v>
       </c>
-      <c r="B22" s="42" t="n">
+      <c r="B22" s="46" t="n">
         <v>0.25</v>
       </c>
-      <c r="C22" s="42" t="n">
+      <c r="C22" s="46" t="n">
         <v>0.05</v>
       </c>
-      <c r="D22" s="42" t="n">
+      <c r="D22" s="46" t="n">
         <v>30000</v>
       </c>
-      <c r="E22" s="42" t="n">
+      <c r="E22" s="46" t="n">
         <v>506.39</v>
       </c>
-      <c r="F22" s="42" t="n">
+      <c r="F22" s="46" t="n">
         <v>574.24</v>
       </c>
-      <c r="G22" s="42" t="n">
+      <c r="G22" s="46" t="n">
         <v>1.234</v>
       </c>
-      <c r="H22" s="42" t="n">
+      <c r="H22" s="46" t="n">
         <v>0.77407</v>
       </c>
-      <c r="I22" s="42" t="n">
+      <c r="I22" s="46" t="n">
         <v>37764.9</v>
       </c>
-      <c r="J22" s="42" t="inlineStr">
+      <c r="J22" s="46" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="K22" s="43" t="inlineStr"/>
+      <c r="K22" s="47" t="inlineStr"/>
     </row>
     <row r="23" ht="15" customHeight="1">
-      <c r="A23" s="42" t="n">
+      <c r="A23" s="46" t="n">
         <v>19</v>
       </c>
-      <c r="B23" s="42" t="n">
+      <c r="B23" s="46" t="n">
         <v>0.25</v>
       </c>
-      <c r="C23" s="42" t="n">
+      <c r="C23" s="46" t="n">
         <v>0.1</v>
       </c>
-      <c r="D23" s="42" t="n">
+      <c r="D23" s="46" t="n">
         <v>5000</v>
       </c>
-      <c r="E23" s="42" t="n">
+      <c r="E23" s="46" t="n">
         <v>539.17</v>
       </c>
-      <c r="F23" s="42" t="n">
+      <c r="F23" s="46" t="n">
         <v>772.3</v>
       </c>
-      <c r="G23" s="42" t="n">
+      <c r="G23" s="46" t="n">
         <v>0.2028</v>
       </c>
-      <c r="H23" s="42" t="n">
+      <c r="H23" s="46" t="n">
         <v>0.03744</v>
       </c>
-      <c r="I23" s="42" t="n">
+      <c r="I23" s="46" t="n">
         <v>37764.9</v>
       </c>
-      <c r="J23" s="42" t="inlineStr">
+      <c r="J23" s="46" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="K23" s="43" t="inlineStr"/>
+      <c r="K23" s="47" t="inlineStr"/>
     </row>
     <row r="24" ht="15" customHeight="1">
-      <c r="A24" s="42" t="n">
+      <c r="A24" s="46" t="n">
         <v>20</v>
       </c>
-      <c r="B24" s="42" t="n">
+      <c r="B24" s="46" t="n">
         <v>0.25</v>
       </c>
-      <c r="C24" s="42" t="n">
+      <c r="C24" s="46" t="n">
         <v>0.1</v>
       </c>
-      <c r="D24" s="42" t="n">
+      <c r="D24" s="46" t="n">
         <v>10000</v>
       </c>
-      <c r="E24" s="42" t="n">
+      <c r="E24" s="46" t="n">
         <v>519.63</v>
       </c>
-      <c r="F24" s="42" t="n">
+      <c r="F24" s="46" t="n">
         <v>673.22</v>
       </c>
-      <c r="G24" s="42" t="n">
+      <c r="G24" s="46" t="n">
         <v>0.4057</v>
       </c>
-      <c r="H24" s="42" t="n">
+      <c r="H24" s="46" t="n">
         <v>0.11728</v>
       </c>
-      <c r="I24" s="42" t="n">
+      <c r="I24" s="46" t="n">
         <v>37764.9</v>
       </c>
-      <c r="J24" s="42" t="inlineStr">
+      <c r="J24" s="46" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="K24" s="43" t="inlineStr"/>
+      <c r="K24" s="47" t="inlineStr"/>
     </row>
     <row r="25" ht="15" customHeight="1">
-      <c r="A25" s="42" t="n">
+      <c r="A25" s="46" t="n">
         <v>21</v>
       </c>
-      <c r="B25" s="42" t="n">
+      <c r="B25" s="46" t="n">
         <v>0.25</v>
       </c>
-      <c r="C25" s="42" t="n">
+      <c r="C25" s="46" t="n">
         <v>0.1</v>
       </c>
-      <c r="D25" s="42" t="n">
+      <c r="D25" s="46" t="n">
         <v>15000</v>
       </c>
-      <c r="E25" s="42" t="n">
+      <c r="E25" s="46" t="n">
         <v>511.75</v>
       </c>
-      <c r="F25" s="42" t="n">
+      <c r="F25" s="46" t="n">
         <v>622.35</v>
       </c>
-      <c r="G25" s="42" t="n">
+      <c r="G25" s="46" t="n">
         <v>0.6085</v>
       </c>
-      <c r="H25" s="42" t="n">
+      <c r="H25" s="46" t="n">
         <v>0.27748</v>
       </c>
-      <c r="I25" s="42" t="n">
+      <c r="I25" s="46" t="n">
         <v>37764.5</v>
       </c>
-      <c r="J25" s="42" t="inlineStr">
+      <c r="J25" s="46" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="K25" s="43" t="inlineStr"/>
+      <c r="K25" s="47" t="inlineStr"/>
     </row>
     <row r="26" ht="15" customHeight="1">
-      <c r="A26" s="42" t="n">
+      <c r="A26" s="46" t="n">
         <v>22</v>
       </c>
-      <c r="B26" s="42" t="n">
+      <c r="B26" s="46" t="n">
         <v>0.25</v>
       </c>
-      <c r="C26" s="42" t="n">
+      <c r="C26" s="46" t="n">
         <v>0.1</v>
       </c>
-      <c r="D26" s="42" t="n">
+      <c r="D26" s="46" t="n">
         <v>20000</v>
       </c>
-      <c r="E26" s="42" t="n">
+      <c r="E26" s="46" t="n">
         <v>509.82</v>
       </c>
-      <c r="F26" s="42" t="n">
+      <c r="F26" s="46" t="n">
         <v>599.35</v>
       </c>
-      <c r="G26" s="42" t="n">
+      <c r="G26" s="46" t="n">
         <v>0.8113</v>
       </c>
-      <c r="H26" s="42" t="n">
+      <c r="H26" s="46" t="n">
         <v>0.41921</v>
       </c>
-      <c r="I26" s="42" t="n">
+      <c r="I26" s="46" t="n">
         <v>37764.8</v>
       </c>
-      <c r="J26" s="42" t="inlineStr">
+      <c r="J26" s="46" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="K26" s="43" t="inlineStr"/>
+      <c r="K26" s="47" t="inlineStr"/>
     </row>
     <row r="27" ht="15" customHeight="1">
-      <c r="A27" s="42" t="n">
+      <c r="A27" s="46" t="n">
         <v>23</v>
       </c>
-      <c r="B27" s="42" t="n">
+      <c r="B27" s="46" t="n">
         <v>0.25</v>
       </c>
-      <c r="C27" s="42" t="n">
+      <c r="C27" s="46" t="n">
         <v>0.1</v>
       </c>
-      <c r="D27" s="42" t="n">
+      <c r="D27" s="46" t="n">
         <v>25000</v>
       </c>
-      <c r="E27" s="42" t="n">
+      <c r="E27" s="46" t="n">
         <v>507.86</v>
       </c>
-      <c r="F27" s="42" t="n">
+      <c r="F27" s="46" t="n">
         <v>586.09</v>
       </c>
-      <c r="G27" s="42" t="n">
+      <c r="G27" s="46" t="n">
         <v>1.0142</v>
       </c>
-      <c r="H27" s="42" t="n">
+      <c r="H27" s="46" t="n">
         <v>0.55332</v>
       </c>
-      <c r="I27" s="42" t="n">
+      <c r="I27" s="46" t="n">
         <v>37764.9</v>
       </c>
-      <c r="J27" s="42" t="inlineStr">
+      <c r="J27" s="46" t="inlineStr">
         <is>
           <t>FIXED</t>
         </is>
       </c>
-      <c r="K27" s="43" t="inlineStr">
+      <c r="K27" s="47" t="inlineStr">
         <is>
           <t>Re-run 2026-10-04: transient (50 steps, dt=1e-4s) then Steady; converged cleanly</t>
         </is>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1">
-      <c r="A28" s="42" t="n">
+      <c r="A28" s="46" t="n">
         <v>24</v>
       </c>
-      <c r="B28" s="42" t="n">
+      <c r="B28" s="46" t="n">
         <v>0.25</v>
       </c>
-      <c r="C28" s="42" t="n">
+      <c r="C28" s="46" t="n">
         <v>0.1</v>
       </c>
-      <c r="D28" s="42" t="n">
+      <c r="D28" s="46" t="n">
         <v>30000</v>
       </c>
-      <c r="E28" s="42" t="n">
+      <c r="E28" s="46" t="n">
         <v>506.54</v>
       </c>
-      <c r="F28" s="42" t="n">
+      <c r="F28" s="46" t="n">
         <v>573.4</v>
       </c>
-      <c r="G28" s="42" t="n">
+      <c r="G28" s="46" t="n">
         <v>1.217</v>
       </c>
-      <c r="H28" s="42" t="n">
+      <c r="H28" s="46" t="n">
         <v>0.80392</v>
       </c>
-      <c r="I28" s="42" t="n">
+      <c r="I28" s="46" t="n">
         <v>37765</v>
       </c>
-      <c r="J28" s="42" t="inlineStr">
+      <c r="J28" s="46" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="K28" s="43" t="inlineStr"/>
+      <c r="K28" s="47" t="inlineStr"/>
     </row>
     <row r="29" ht="15" customHeight="1">
-      <c r="A29" s="42" t="n">
+      <c r="A29" s="46" t="n">
         <v>25</v>
       </c>
-      <c r="B29" s="42" t="n">
+      <c r="B29" s="46" t="n">
         <v>0.25</v>
       </c>
-      <c r="C29" s="42" t="n">
+      <c r="C29" s="46" t="n">
         <v>0.15</v>
       </c>
-      <c r="D29" s="42" t="n">
+      <c r="D29" s="46" t="n">
         <v>5000</v>
       </c>
-      <c r="E29" s="42" t="n">
+      <c r="E29" s="46" t="n">
         <v>539.66</v>
       </c>
-      <c r="F29" s="42" t="n">
+      <c r="F29" s="46" t="n">
         <v>772.28</v>
       </c>
-      <c r="G29" s="42" t="n">
+      <c r="G29" s="46" t="n">
         <v>0.2003</v>
       </c>
-      <c r="H29" s="42" t="n">
+      <c r="H29" s="46" t="n">
         <v>0.03745</v>
       </c>
-      <c r="I29" s="42" t="n">
+      <c r="I29" s="46" t="n">
         <v>37764.9</v>
       </c>
-      <c r="J29" s="42" t="inlineStr">
+      <c r="J29" s="46" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="K29" s="43" t="inlineStr"/>
+      <c r="K29" s="47" t="inlineStr"/>
     </row>
     <row r="30" ht="15" customHeight="1">
-      <c r="A30" s="42" t="n">
+      <c r="A30" s="46" t="n">
         <v>26</v>
       </c>
-      <c r="B30" s="42" t="n">
+      <c r="B30" s="46" t="n">
         <v>0.25</v>
       </c>
-      <c r="C30" s="42" t="n">
+      <c r="C30" s="46" t="n">
         <v>0.15</v>
       </c>
-      <c r="D30" s="42" t="n">
+      <c r="D30" s="46" t="n">
         <v>10000</v>
       </c>
-      <c r="E30" s="42" t="n">
+      <c r="E30" s="46" t="n">
         <v>512.65</v>
       </c>
-      <c r="F30" s="42" t="n">
+      <c r="F30" s="46" t="n">
         <v>659.64</v>
       </c>
-      <c r="G30" s="42" t="n">
+      <c r="G30" s="46" t="n">
         <v>0.4007</v>
       </c>
-      <c r="H30" s="42" t="n">
+      <c r="H30" s="46" t="n">
         <v>0.17827</v>
       </c>
-      <c r="I30" s="42" t="n">
+      <c r="I30" s="46" t="n">
         <v>37764.8</v>
       </c>
-      <c r="J30" s="42" t="inlineStr">
+      <c r="J30" s="46" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="K30" s="43" t="inlineStr"/>
+      <c r="K30" s="47" t="inlineStr"/>
     </row>
     <row r="31" ht="15" customHeight="1">
-      <c r="A31" s="42" t="n">
+      <c r="A31" s="46" t="n">
         <v>27</v>
       </c>
-      <c r="B31" s="42" t="n">
+      <c r="B31" s="46" t="n">
         <v>0.25</v>
       </c>
-      <c r="C31" s="42" t="n">
+      <c r="C31" s="46" t="n">
         <v>0.15</v>
       </c>
-      <c r="D31" s="42" t="n">
+      <c r="D31" s="46" t="n">
         <v>15000</v>
       </c>
-      <c r="E31" s="42" t="n">
+      <c r="E31" s="46" t="n">
         <v>512.8099999999999</v>
       </c>
-      <c r="F31" s="42" t="n">
+      <c r="F31" s="46" t="n">
         <v>622.58</v>
       </c>
-      <c r="G31" s="42" t="n">
+      <c r="G31" s="46" t="n">
         <v>0.601</v>
       </c>
-      <c r="H31" s="42" t="n">
+      <c r="H31" s="46" t="n">
         <v>0.27715</v>
       </c>
-      <c r="I31" s="42" t="n">
+      <c r="I31" s="46" t="n">
         <v>37764.5</v>
       </c>
-      <c r="J31" s="42" t="inlineStr">
+      <c r="J31" s="46" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="K31" s="43" t="inlineStr"/>
+      <c r="K31" s="47" t="inlineStr"/>
     </row>
     <row r="32" ht="15" customHeight="1">
-      <c r="A32" s="42" t="n">
+      <c r="A32" s="46" t="n">
         <v>28</v>
       </c>
-      <c r="B32" s="42" t="n">
+      <c r="B32" s="46" t="n">
         <v>0.25</v>
       </c>
-      <c r="C32" s="42" t="n">
+      <c r="C32" s="46" t="n">
         <v>0.15</v>
       </c>
-      <c r="D32" s="42" t="n">
+      <c r="D32" s="46" t="n">
         <v>20000</v>
       </c>
-      <c r="E32" s="42" t="n">
+      <c r="E32" s="46" t="n">
         <v>509.95</v>
       </c>
-      <c r="F32" s="42" t="n">
+      <c r="F32" s="46" t="n">
         <v>601.83</v>
       </c>
-      <c r="G32" s="42" t="n">
+      <c r="G32" s="46" t="n">
         <v>0.8014</v>
       </c>
-      <c r="H32" s="42" t="n">
+      <c r="H32" s="46" t="n">
         <v>0.38019</v>
       </c>
-      <c r="I32" s="42" t="n">
+      <c r="I32" s="46" t="n">
         <v>37764.9</v>
       </c>
-      <c r="J32" s="42" t="inlineStr">
+      <c r="J32" s="46" t="inlineStr">
         <is>
           <t>FIXED</t>
         </is>
       </c>
-      <c r="K32" s="43" t="inlineStr">
+      <c r="K32" s="47" t="inlineStr">
         <is>
           <t>Re-run 2026-10-04: same transient-then-Steady fix; converged cleanly</t>
         </is>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1">
-      <c r="A33" s="42" t="n">
+      <c r="A33" s="46" t="n">
         <v>29</v>
       </c>
-      <c r="B33" s="42" t="n">
+      <c r="B33" s="46" t="n">
         <v>0.25</v>
       </c>
-      <c r="C33" s="42" t="n">
+      <c r="C33" s="46" t="n">
         <v>0.15</v>
       </c>
-      <c r="D33" s="42" t="n">
+      <c r="D33" s="46" t="n">
         <v>25000</v>
       </c>
-      <c r="E33" s="42" t="n">
+      <c r="E33" s="46" t="n">
         <v>507.96</v>
       </c>
-      <c r="F33" s="42" t="n">
+      <c r="F33" s="46" t="n">
         <v>584.08</v>
       </c>
-      <c r="G33" s="42" t="n">
+      <c r="G33" s="46" t="n">
         <v>1.0017</v>
       </c>
-      <c r="H33" s="42" t="n">
+      <c r="H33" s="46" t="n">
         <v>0.61978</v>
       </c>
-      <c r="I33" s="42" t="n">
+      <c r="I33" s="46" t="n">
         <v>37764.7</v>
       </c>
-      <c r="J33" s="42" t="inlineStr">
+      <c r="J33" s="46" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="K33" s="43" t="inlineStr"/>
+      <c r="K33" s="47" t="inlineStr"/>
     </row>
     <row r="34" ht="15" customHeight="1">
-      <c r="A34" s="44" t="n">
+      <c r="A34" s="46" t="n">
         <v>30</v>
       </c>
-      <c r="B34" s="44" t="n">
+      <c r="B34" s="46" t="n">
         <v>0.25</v>
       </c>
-      <c r="C34" s="44" t="n">
+      <c r="C34" s="46" t="n">
         <v>0.15</v>
       </c>
-      <c r="D34" s="44" t="n">
+      <c r="D34" s="46" t="n">
         <v>30000</v>
       </c>
-      <c r="E34" s="44" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F34" s="44" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G34" s="44" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H34" s="44" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I34" s="44" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J34" s="44" t="inlineStr">
-        <is>
-          <t>NOT RUN</t>
-        </is>
-      </c>
-      <c r="K34" s="45" t="inlineStr">
-        <is>
-          <t>No data in this export — remaining, not yet re-run</t>
+      <c r="E34" s="46" t="n">
+        <v>506.53</v>
+      </c>
+      <c r="F34" s="46" t="n">
+        <v>573.73</v>
+      </c>
+      <c r="G34" s="46" t="n">
+        <v>1.2217</v>
+      </c>
+      <c r="H34" s="46" t="n">
+        <v>0.81645</v>
+      </c>
+      <c r="I34" s="46" t="n">
+        <v>37765</v>
+      </c>
+      <c r="J34" s="48" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="K34" s="49" t="inlineStr">
+        <is>
+          <t>Run 54 — re-run 2026-10-07 (transient-then-Steady fix); now converged cleanly</t>
         </is>
       </c>
     </row>
@@ -9251,7 +9265,7 @@
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="27" t="inlineStr">
         <is>
-          <t>Section 2 — Promoter-Size Comparison (Stage 2: tp/dpo=0.05 fixed)</t>
+          <t>Section 2 — Promoter-Size Comparison (Stage 2: tp/dpo=0.05 fixed) — CONFIRMED, 6/6 valid in every group</t>
         </is>
       </c>
       <c r="B38" s="13" t="n"/>
@@ -9318,240 +9332,237 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="42" t="n">
+      <c r="A40" s="46" t="n">
         <v>5000</v>
       </c>
-      <c r="B40" s="42" t="n">
+      <c r="B40" s="46" t="n">
         <v>0.96223</v>
       </c>
-      <c r="C40" s="42" t="n">
+      <c r="C40" s="46" t="n">
         <v>1.00387</v>
       </c>
-      <c r="D40" s="42" t="n">
+      <c r="D40" s="46" t="n">
         <v>1.05945</v>
       </c>
-      <c r="E40" s="42" t="n">
+      <c r="E40" s="46" t="n">
         <v>1.20294</v>
       </c>
-      <c r="F40" s="42" t="n">
+      <c r="F40" s="46" t="n">
         <v>1.25322</v>
       </c>
-      <c r="G40" s="42" t="n">
+      <c r="G40" s="46" t="n">
         <v>1.30761</v>
       </c>
-      <c r="H40" s="42" t="n">
+      <c r="H40" s="46" t="n">
         <v>1.21847</v>
       </c>
-      <c r="I40" s="42" t="n">
+      <c r="I40" s="46" t="n">
         <v>1.2516</v>
       </c>
-      <c r="J40" s="42" t="n">
+      <c r="J40" s="46" t="n">
         <v>1.28268</v>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="42" t="n">
+      <c r="A41" s="46" t="n">
         <v>10000</v>
       </c>
-      <c r="B41" s="42" t="n">
+      <c r="B41" s="46" t="n">
         <v>0.89286</v>
       </c>
-      <c r="C41" s="42" t="n">
+      <c r="C41" s="46" t="n">
         <v>0.92806</v>
       </c>
-      <c r="D41" s="42" t="n">
+      <c r="D41" s="46" t="n">
         <v>1.16817</v>
       </c>
-      <c r="E41" s="42" t="n">
+      <c r="E41" s="46" t="n">
         <v>1.09948</v>
       </c>
-      <c r="F41" s="42" t="n">
+      <c r="F41" s="46" t="n">
         <v>1.13054</v>
       </c>
-      <c r="G41" s="42" t="n">
+      <c r="G41" s="46" t="n">
         <v>1.18763</v>
       </c>
-      <c r="H41" s="42" t="n">
+      <c r="H41" s="46" t="n">
         <v>1.1418</v>
       </c>
-      <c r="I41" s="42" t="n">
+      <c r="I41" s="46" t="n">
         <v>1.15903</v>
       </c>
-      <c r="J41" s="42" t="n">
+      <c r="J41" s="46" t="n">
         <v>1.12766</v>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="42" t="n">
+      <c r="A42" s="46" t="n">
         <v>15000</v>
       </c>
-      <c r="B42" s="42" t="n">
+      <c r="B42" s="46" t="n">
         <v>0.86965</v>
       </c>
-      <c r="C42" s="42" t="n">
+      <c r="C42" s="46" t="n">
         <v>0.90156</v>
       </c>
-      <c r="D42" s="34">
-        <f>NA()</f>
-        <v/>
-      </c>
-      <c r="E42" s="42" t="n">
+      <c r="D42" s="46" t="n">
+        <v>0.9429</v>
+      </c>
+      <c r="E42" s="46" t="n">
         <v>1.06637</v>
       </c>
-      <c r="F42" s="42" t="n">
+      <c r="F42" s="46" t="n">
         <v>1.09106</v>
       </c>
-      <c r="G42" s="34">
-        <f>NA()</f>
-        <v/>
-      </c>
-      <c r="H42" s="42" t="n">
+      <c r="G42" s="46" t="n">
+        <v>1.12017</v>
+      </c>
+      <c r="H42" s="46" t="n">
         <v>1.11719</v>
       </c>
-      <c r="I42" s="42" t="n">
+      <c r="I42" s="46" t="n">
         <v>1.12941</v>
       </c>
-      <c r="J42" s="34">
-        <f>NA()</f>
-        <v/>
+      <c r="J42" s="46" t="n">
+        <v>1.14234</v>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="42" t="n">
+      <c r="A43" s="46" t="n">
         <v>20000</v>
       </c>
-      <c r="B43" s="42" t="n">
+      <c r="B43" s="46" t="n">
         <v>0.88069</v>
       </c>
-      <c r="C43" s="42" t="n">
+      <c r="C43" s="46" t="n">
         <v>0.91301</v>
       </c>
-      <c r="D43" s="42" t="n">
+      <c r="D43" s="46" t="n">
         <v>1.06595</v>
       </c>
-      <c r="E43" s="42" t="n">
+      <c r="E43" s="46" t="n">
         <v>1.07778</v>
       </c>
-      <c r="F43" s="42" t="n">
+      <c r="F43" s="46" t="n">
         <v>1.10065</v>
       </c>
-      <c r="G43" s="42" t="n">
+      <c r="G43" s="46" t="n">
         <v>1.15052</v>
       </c>
-      <c r="H43" s="42" t="n">
+      <c r="H43" s="46" t="n">
         <v>1.1244</v>
       </c>
-      <c r="I43" s="42" t="n">
+      <c r="I43" s="46" t="n">
         <v>1.13455</v>
       </c>
-      <c r="J43" s="42" t="n">
+      <c r="J43" s="46" t="n">
         <v>1.12628</v>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="42" t="n">
+      <c r="A44" s="46" t="n">
         <v>25000</v>
       </c>
-      <c r="B44" s="42" t="n">
+      <c r="B44" s="46" t="n">
         <v>0.90709</v>
       </c>
-      <c r="C44" s="42" t="n">
+      <c r="C44" s="46" t="n">
         <v>0.94098</v>
       </c>
-      <c r="D44" s="42" t="n">
+      <c r="D44" s="46" t="n">
         <v>1.04956</v>
       </c>
-      <c r="E44" s="42" t="n">
+      <c r="E44" s="46" t="n">
         <v>1.08219</v>
       </c>
-      <c r="F44" s="42" t="n">
+      <c r="F44" s="46" t="n">
         <v>1.10437</v>
       </c>
-      <c r="G44" s="42" t="n">
+      <c r="G44" s="46" t="n">
         <v>1.15066</v>
       </c>
-      <c r="H44" s="42" t="n">
+      <c r="H44" s="46" t="n">
         <v>1.11794</v>
       </c>
-      <c r="I44" s="42" t="n">
+      <c r="I44" s="46" t="n">
         <v>1.12699</v>
       </c>
-      <c r="J44" s="42" t="n">
+      <c r="J44" s="46" t="n">
         <v>1.13225</v>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="42" t="n">
+      <c r="A45" s="46" t="n">
         <v>30000</v>
       </c>
-      <c r="B45" s="42" t="n">
+      <c r="B45" s="46" t="n">
         <v>0.9241</v>
       </c>
-      <c r="C45" s="42" t="n">
+      <c r="C45" s="46" t="n">
         <v>0.95941</v>
       </c>
-      <c r="D45" s="42" t="n">
+      <c r="D45" s="46" t="n">
         <v>1.03505</v>
       </c>
-      <c r="E45" s="42" t="n">
+      <c r="E45" s="46" t="n">
         <v>1.08203</v>
       </c>
-      <c r="F45" s="42" t="n">
+      <c r="F45" s="46" t="n">
         <v>1.10424</v>
       </c>
-      <c r="G45" s="42" t="n">
+      <c r="G45" s="46" t="n">
         <v>1.14381</v>
       </c>
-      <c r="H45" s="42" t="n">
+      <c r="H45" s="46" t="n">
         <v>1.11088</v>
       </c>
-      <c r="I45" s="42" t="n">
+      <c r="I45" s="46" t="n">
         <v>1.1196</v>
       </c>
-      <c r="J45" s="42" t="n">
+      <c r="J45" s="46" t="n">
         <v>1.13075</v>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="43" t="inlineStr">
+      <c r="A47" s="47" t="inlineStr">
         <is>
           <t>mean PEC (dpo/dti=0.15)</t>
         </is>
       </c>
-      <c r="B47" s="43" t="inlineStr">
+      <c r="B47" s="47" t="inlineStr">
         <is>
           <t>1.1384  (6/6 valid)</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="43" t="inlineStr">
+      <c r="A48" s="47" t="inlineStr">
         <is>
           <t>mean PEC (dpo/dti=0.2)</t>
         </is>
       </c>
-      <c r="B48" s="43" t="inlineStr">
+      <c r="B48" s="47" t="inlineStr">
         <is>
           <t>1.1535  (6/6 valid)</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="43" t="inlineStr">
-        <is>
-          <t>mean PEC (dpo/dti=0.25)</t>
-        </is>
-      </c>
-      <c r="B49" s="43" t="inlineStr">
-        <is>
-          <t>1.1599  (5/6 valid)</t>
+      <c r="A49" s="50" t="inlineStr">
+        <is>
+          <t>mean PEC (dpo/dti=0.25)  &lt;-- WINNER</t>
+        </is>
+      </c>
+      <c r="B49" s="50" t="inlineStr">
+        <is>
+          <t>1.1570  (6/6 valid)</t>
         </is>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="27" t="inlineStr">
         <is>
-          <t>Section 3 — Wall-Thickness Comparison (Stage 3: dpo/dti=0.25 fixed)</t>
+          <t>Section 3 — Wall-Thickness Comparison (Stage 3: dpo/dti=0.25 fixed) — CONFIRMED, 6/6 valid in every group</t>
         </is>
       </c>
       <c r="B51" s="13" t="n"/>
@@ -9618,236 +9629,230 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="42" t="n">
+      <c r="A53" s="46" t="n">
         <v>5000</v>
       </c>
-      <c r="B53" s="42" t="n">
+      <c r="B53" s="46" t="n">
         <v>1.05945</v>
       </c>
-      <c r="C53" s="42" t="n">
+      <c r="C53" s="46" t="n">
         <v>1.06354</v>
       </c>
-      <c r="D53" s="42" t="n">
+      <c r="D53" s="46" t="n">
         <v>1.06924</v>
       </c>
-      <c r="E53" s="42" t="n">
+      <c r="E53" s="46" t="n">
         <v>1.30761</v>
       </c>
-      <c r="F53" s="42" t="n">
+      <c r="F53" s="46" t="n">
         <v>1.30456</v>
       </c>
-      <c r="G53" s="42" t="n">
+      <c r="G53" s="46" t="n">
         <v>1.30657</v>
       </c>
-      <c r="H53" s="42" t="n">
+      <c r="H53" s="46" t="n">
         <v>1.28268</v>
       </c>
-      <c r="I53" s="42" t="n">
+      <c r="I53" s="46" t="n">
         <v>1.27804</v>
       </c>
-      <c r="J53" s="42" t="n">
+      <c r="J53" s="46" t="n">
         <v>1.27774</v>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="42" t="n">
+      <c r="A54" s="46" t="n">
         <v>10000</v>
       </c>
-      <c r="B54" s="42" t="n">
+      <c r="B54" s="46" t="n">
         <v>1.16817</v>
       </c>
-      <c r="C54" s="42" t="n">
+      <c r="C54" s="46" t="n">
         <v>0.97993</v>
       </c>
-      <c r="D54" s="42" t="n">
+      <c r="D54" s="46" t="n">
         <v>1.50508</v>
       </c>
-      <c r="E54" s="42" t="n">
+      <c r="E54" s="46" t="n">
         <v>1.18763</v>
       </c>
-      <c r="F54" s="42" t="n">
+      <c r="F54" s="46" t="n">
         <v>1.16579</v>
       </c>
-      <c r="G54" s="42" t="n">
+      <c r="G54" s="46" t="n">
         <v>1.23395</v>
       </c>
-      <c r="H54" s="42" t="n">
+      <c r="H54" s="46" t="n">
         <v>1.12766</v>
       </c>
-      <c r="I54" s="42" t="n">
+      <c r="I54" s="46" t="n">
         <v>1.17369</v>
       </c>
-      <c r="J54" s="42" t="n">
+      <c r="J54" s="46" t="n">
         <v>1.07674</v>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="42" t="n">
+      <c r="A55" s="46" t="n">
         <v>15000</v>
       </c>
-      <c r="B55" s="34">
-        <f>NA()</f>
-        <v/>
-      </c>
-      <c r="C55" s="42" t="n">
+      <c r="B55" s="46" t="n">
+        <v>0.9429</v>
+      </c>
+      <c r="C55" s="46" t="n">
         <v>1.12924</v>
       </c>
-      <c r="D55" s="42" t="n">
+      <c r="D55" s="46" t="n">
         <v>1.13328</v>
       </c>
-      <c r="E55" s="34">
-        <f>NA()</f>
-        <v/>
-      </c>
-      <c r="F55" s="42" t="n">
+      <c r="E55" s="46" t="n">
+        <v>1.12017</v>
+      </c>
+      <c r="F55" s="46" t="n">
         <v>1.15911</v>
       </c>
-      <c r="G55" s="42" t="n">
+      <c r="G55" s="46" t="n">
         <v>1.16327</v>
       </c>
-      <c r="H55" s="34">
-        <f>NA()</f>
-        <v/>
-      </c>
-      <c r="I55" s="42" t="n">
+      <c r="H55" s="46" t="n">
+        <v>1.14234</v>
+      </c>
+      <c r="I55" s="46" t="n">
         <v>1.11309</v>
       </c>
-      <c r="J55" s="42" t="n">
+      <c r="J55" s="46" t="n">
         <v>1.11575</v>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="42" t="n">
+      <c r="A56" s="46" t="n">
         <v>20000</v>
       </c>
-      <c r="B56" s="42" t="n">
+      <c r="B56" s="46" t="n">
         <v>1.06595</v>
       </c>
-      <c r="C56" s="42" t="n">
+      <c r="C56" s="46" t="n">
         <v>1.05751</v>
       </c>
-      <c r="D56" s="42" t="n">
+      <c r="D56" s="46" t="n">
         <v>0.96427</v>
       </c>
-      <c r="E56" s="42" t="n">
+      <c r="E56" s="46" t="n">
         <v>1.15052</v>
       </c>
-      <c r="F56" s="42" t="n">
+      <c r="F56" s="46" t="n">
         <v>1.15727</v>
       </c>
-      <c r="G56" s="42" t="n">
+      <c r="G56" s="46" t="n">
         <v>1.12854</v>
       </c>
-      <c r="H56" s="42" t="n">
+      <c r="H56" s="46" t="n">
         <v>1.12628</v>
       </c>
-      <c r="I56" s="42" t="n">
+      <c r="I56" s="46" t="n">
         <v>1.1359</v>
       </c>
-      <c r="J56" s="42" t="n">
+      <c r="J56" s="46" t="n">
         <v>1.14232</v>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="42" t="n">
+      <c r="A57" s="46" t="n">
         <v>25000</v>
       </c>
-      <c r="B57" s="42" t="n">
+      <c r="B57" s="46" t="n">
         <v>1.04956</v>
       </c>
-      <c r="C57" s="42" t="n">
+      <c r="C57" s="46" t="n">
         <v>0.98776</v>
       </c>
-      <c r="D57" s="42" t="n">
+      <c r="D57" s="46" t="n">
         <v>1.11242</v>
       </c>
-      <c r="E57" s="42" t="n">
+      <c r="E57" s="46" t="n">
         <v>1.15066</v>
       </c>
-      <c r="F57" s="42" t="n">
+      <c r="F57" s="46" t="n">
         <v>1.13014</v>
       </c>
-      <c r="G57" s="42" t="n">
+      <c r="G57" s="46" t="n">
         <v>1.15933</v>
       </c>
-      <c r="H57" s="42" t="n">
+      <c r="H57" s="46" t="n">
         <v>1.13225</v>
       </c>
-      <c r="I57" s="42" t="n">
+      <c r="I57" s="46" t="n">
         <v>1.13479</v>
       </c>
-      <c r="J57" s="42" t="n">
+      <c r="J57" s="46" t="n">
         <v>1.11888</v>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="42" t="n">
+      <c r="A58" s="46" t="n">
         <v>30000</v>
       </c>
-      <c r="B58" s="42" t="n">
+      <c r="B58" s="46" t="n">
         <v>1.03505</v>
       </c>
-      <c r="C58" s="42" t="n">
+      <c r="C58" s="46" t="n">
         <v>1.08141</v>
       </c>
-      <c r="D58" s="34">
-        <f>NA()</f>
-        <v/>
-      </c>
-      <c r="E58" s="42" t="n">
+      <c r="D58" s="46" t="n">
+        <v>1.06906</v>
+      </c>
+      <c r="E58" s="46" t="n">
         <v>1.14381</v>
       </c>
-      <c r="F58" s="42" t="n">
+      <c r="F58" s="46" t="n">
         <v>1.15889</v>
       </c>
-      <c r="G58" s="34">
-        <f>NA()</f>
-        <v/>
-      </c>
-      <c r="H58" s="42" t="n">
+      <c r="G58" s="46" t="n">
+        <v>1.15337</v>
+      </c>
+      <c r="H58" s="46" t="n">
         <v>1.13075</v>
       </c>
-      <c r="I58" s="42" t="n">
+      <c r="I58" s="46" t="n">
         <v>1.12905</v>
       </c>
-      <c r="J58" s="34">
-        <f>NA()</f>
-        <v/>
+      <c r="J58" s="46" t="n">
+        <v>1.12798</v>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="43" t="inlineStr">
+      <c r="A60" s="47" t="inlineStr">
         <is>
           <t>mean PEC (tp/dpo=0.05)</t>
         </is>
       </c>
-      <c r="B60" s="43" t="inlineStr">
-        <is>
-          <t>1.1599  (5/6 valid)</t>
+      <c r="B60" s="47" t="inlineStr">
+        <is>
+          <t>1.1570  (6/6 valid)</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="43" t="inlineStr">
-        <is>
-          <t>mean PEC (tp/dpo=0.1)</t>
-        </is>
-      </c>
-      <c r="B61" s="43" t="inlineStr">
+      <c r="A61" s="50" t="inlineStr">
+        <is>
+          <t>mean PEC (tp/dpo=0.1)  &lt;-- WINNER</t>
+        </is>
+      </c>
+      <c r="B61" s="50" t="inlineStr">
         <is>
           <t>1.1608  (6/6 valid)</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="43" t="inlineStr">
+      <c r="A62" s="47" t="inlineStr">
         <is>
           <t>mean PEC (tp/dpo=0.15)</t>
         </is>
       </c>
-      <c r="B62" s="43" t="inlineStr">
-        <is>
-          <t>1.1463  (5/6 valid)</t>
+      <c r="B62" s="47" t="inlineStr">
+        <is>
+          <t>1.1432  (6/6 valid)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add methodology note on transient-to-steady divergence recovery
Documents the pseudo-transient continuation justification (Kelley &
Keyes 1998) with explicit proven-vs-practitioner-consensus framing,
plus references to pull deeper evidence from before thesis submission.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DUewHsWD72fWTrA8cwVfXx
</commit_message>
<xml_diff>
--- a/Parameter_Run_Tracking_Table.xlsx
+++ b/Parameter_Run_Tracking_Table.xlsx
@@ -2396,7 +2396,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F93"/>
+  <dimension ref="A1:F106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3951,12 +3951,158 @@
       <c r="E93" s="13" t="n"/>
       <c r="F93" s="14" t="n"/>
     </row>
+    <row r="95" ht="20" customHeight="1">
+      <c r="A95" s="15" t="inlineStr">
+        <is>
+          <t>Methodology Note — Transient-then-Steady Divergence Recovery (used for Runs 39, 47, 52, 54 and Stage-4 nanofluid re-runs)</t>
+        </is>
+      </c>
+      <c r="B95" s="15" t="n"/>
+      <c r="C95" s="15" t="n"/>
+      <c r="D95" s="15" t="n"/>
+      <c r="E95" s="15" t="n"/>
+      <c r="F95" s="15" t="n"/>
+    </row>
+    <row r="96" ht="46" customHeight="1">
+      <c r="A96" s="7" t="inlineStr">
+        <is>
+          <t>Several runs diverged in direct Steady mode due to reversed flow at the pressure outlet — a known failure mode for Newton-type steady solvers. Fix: run a short Transient burst (small dt, 50 timesteps, 50 max iterations/step) purely to let the flow settle direction, verify with 3 checks (zero reversed-flow messages / balanced mdot_in-mdot_out / flattened tau_wall), then switch Solver &gt; Time to Steady WITHOUT re-initializing and continue.</t>
+        </is>
+      </c>
+      <c r="B96" s="7" t="n"/>
+      <c r="C96" s="7" t="n"/>
+      <c r="D96" s="7" t="n"/>
+      <c r="E96" s="7" t="n"/>
+      <c r="F96" s="7" t="n"/>
+    </row>
+    <row r="98" ht="18" customHeight="1">
+      <c r="A98" s="3" t="inlineStr">
+        <is>
+          <t>What is proven vs. what is practitioner consensus — be precise about this if asked by advisor/committee</t>
+        </is>
+      </c>
+      <c r="B98" s="3" t="n"/>
+      <c r="C98" s="3" t="n"/>
+      <c r="D98" s="3" t="n"/>
+      <c r="E98" s="3" t="n"/>
+      <c r="F98" s="3" t="n"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="4" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="B99" s="4" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="C99" s="4" t="inlineStr">
+        <is>
+          <t>Reference / where to pull evidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" ht="70" customHeight="1">
+      <c r="A100" s="5" t="inlineStr">
+        <is>
+          <t>The underlying principle (bridging a stalled/diverged steady solve with a short artificial time integration, then growing the timestep back toward steady) is a real, peer-reviewed numerical method: "pseudo-transient continuation" (PTC / ΨtC).</t>
+        </is>
+      </c>
+      <c r="B100" s="5" t="inlineStr">
+        <is>
+          <t>PROVEN — peer-reviewed</t>
+        </is>
+      </c>
+      <c r="C100" s="5" t="inlineStr">
+        <is>
+          <t>Kelley, C.T. and Keyes, D.E. (1998), "Convergence Analysis of Pseudo-Transient Continuation," SIAM Journal on Numerical Analysis, 35(2), pp.508-523. Also: DTIC/ICASE technical report (1996 preprint) — https://apps.dtic.mil/sti/tr/pdf/ADA314613.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" ht="75" customHeight="1">
+      <c r="A101" s="5" t="inlineStr">
+        <is>
+          <t>The exact workflow ("real Transient burst in Fluent, then switch to Steady, no re-init") as a named, sanctioned ANSYS procedure.</t>
+        </is>
+      </c>
+      <c r="B101" s="5" t="inlineStr">
+        <is>
+          <t>NOT FOUND in official docs — practitioner consensus only</t>
+        </is>
+      </c>
+      <c r="C101" s="5" t="inlineStr">
+        <is>
+          <t>No ANSYS Fluent User's Guide section located stating this exact procedure. Supporting field evidence (forum reports of engineers doing this): ANSYS Innovation Space forum, "Steady state and transient solution" — https://innovationspace.ansys.com/forum/forums/topic/steady-state-and-transient-solution/ ; CFD-Online, "Reversed flow on faces of pressure-outlet" — https://www.cfd-online.com/Forums/fluent/245473-reversed-flow-faces-pressure-outlet.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="46" customHeight="1">
+      <c r="A102" s="5" t="inlineStr">
+        <is>
+          <t>Switching Solver &gt; Time (Transient to Steady) preserves the current flow field as the new starting point, rather than resetting it.</t>
+        </is>
+      </c>
+      <c r="B102" s="5" t="inlineStr">
+        <is>
+          <t>Community-verified, not official-doc-verified</t>
+        </is>
+      </c>
+      <c r="C102" s="5" t="inlineStr">
+        <is>
+          <t>Same two forum threads above — multiple independent reports describing this behavior; no official ANSYS documentation page located yet confirming it explicitly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="103" ht="56" customHeight="1">
+      <c r="A103" s="5" t="inlineStr">
+        <is>
+          <t>Surface Report Plots (mass flow rate in/out, area-weighted average wall shear) are the documented, official way to verify convergence beyond residuals alone.</t>
+        </is>
+      </c>
+      <c r="B103" s="5" t="inlineStr">
+        <is>
+          <t>OFFICIAL — documented</t>
+        </is>
+      </c>
+      <c r="C103" s="5" t="inlineStr">
+        <is>
+          <t>ANSYS FLUENT 12.0 Tutorial Guide, Step 8 "Solution" (surface monitor recommended because default residuals alone may not show true convergence) — https://www.afs.enea.it/project/neptunius/docs/fluent/html/tg/node21.htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" ht="70" customHeight="1">
+      <c r="A105" s="23" t="inlineStr">
+        <is>
+          <t>Defensible framing for presentation: "This is an application of pseudo-transient continuation (Kelley &amp; Keyes, 1998), a peer-reviewed globalization method for stalled Newton-type steady solvers. We applied it only where the steady solver demonstrably failed (reversed flow at the outlet), verified recovery with three independent, measurable, documented criteria (surface report plots per the Fluent Tutorial Guide), and switched to Steady without re-initializing to preserve the fixed field. The specific Fluent implementation detail is supported by consistent field practitioner reports, not an ANSYS manual citation — stated honestly, not oversold."</t>
+        </is>
+      </c>
+      <c r="B105" s="23" t="n"/>
+      <c r="C105" s="23" t="n"/>
+      <c r="D105" s="23" t="n"/>
+      <c r="E105" s="23" t="n"/>
+      <c r="F105" s="23" t="n"/>
+    </row>
+    <row r="106" ht="30" customHeight="1">
+      <c r="A106" s="7" t="inlineStr">
+        <is>
+          <t>TODO before final thesis submission: pull the actual Kelley &amp; Keyes (1998) PDF and cite the specific page/section describing the small-to-large timestep growth strategy; if possible, also locate an official ANSYS Fluent Theory Guide or User Guide passage on pseudo-time-stepping / solution stabilization to strengthen the Fluent-specific link.</t>
+        </is>
+      </c>
+      <c r="B106" s="7" t="n"/>
+      <c r="C106" s="7" t="n"/>
+      <c r="D106" s="7" t="n"/>
+      <c r="E106" s="7" t="n"/>
+      <c r="F106" s="7" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="39">
+  <mergeCells count="44">
     <mergeCell ref="A16:F16"/>
     <mergeCell ref="A84:F84"/>
     <mergeCell ref="A75:F75"/>
     <mergeCell ref="A27:F27"/>
+    <mergeCell ref="A105:F105"/>
     <mergeCell ref="A50:F50"/>
     <mergeCell ref="A18:F18"/>
     <mergeCell ref="A56:F56"/>
@@ -3964,6 +4110,7 @@
     <mergeCell ref="E39:F39"/>
     <mergeCell ref="A55:F55"/>
     <mergeCell ref="B38:D38"/>
+    <mergeCell ref="A95:F95"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="E35:F35"/>
     <mergeCell ref="B37:D37"/>
@@ -3971,10 +4118,12 @@
     <mergeCell ref="A42:F42"/>
     <mergeCell ref="A76:F76"/>
     <mergeCell ref="B40:D40"/>
+    <mergeCell ref="A106:F106"/>
     <mergeCell ref="A4:F4"/>
     <mergeCell ref="E40:F40"/>
     <mergeCell ref="A53:F53"/>
     <mergeCell ref="A72:F72"/>
+    <mergeCell ref="A96:F96"/>
     <mergeCell ref="A52:F52"/>
     <mergeCell ref="A10:F10"/>
     <mergeCell ref="B36:D36"/>
@@ -3988,6 +4137,7 @@
     <mergeCell ref="A64:F64"/>
     <mergeCell ref="A73:F73"/>
     <mergeCell ref="A51:F51"/>
+    <mergeCell ref="A98:F98"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="E37:F37"/>
     <mergeCell ref="A78:F78"/>

</xml_diff>

<commit_message>
Add under-relaxation methodology note to Parameter Legend
Documents under-relaxation as the officially vendor-documented
alternative to the transient-then-steady divergence fix, with ANSYS
Fluent User's Guide and forum references. Flags it as not yet applied
to the recovered runs (39, 47, 52, 54, Stage-4 re-runs) — those were
fixed via the transient method before this alternative was identified.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DUewHsWD72fWTrA8cwVfXx
</commit_message>
<xml_diff>
--- a/Parameter_Run_Tracking_Table.xlsx
+++ b/Parameter_Run_Tracking_Table.xlsx
@@ -185,7 +185,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -344,6 +344,12 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2396,7 +2402,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F106"/>
+  <dimension ref="A1:F120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3957,11 +3963,11 @@
           <t>Methodology Note — Transient-then-Steady Divergence Recovery (used for Runs 39, 47, 52, 54 and Stage-4 nanofluid re-runs)</t>
         </is>
       </c>
-      <c r="B95" s="15" t="n"/>
-      <c r="C95" s="15" t="n"/>
-      <c r="D95" s="15" t="n"/>
-      <c r="E95" s="15" t="n"/>
-      <c r="F95" s="15" t="n"/>
+      <c r="B95" s="13" t="n"/>
+      <c r="C95" s="13" t="n"/>
+      <c r="D95" s="13" t="n"/>
+      <c r="E95" s="13" t="n"/>
+      <c r="F95" s="14" t="n"/>
     </row>
     <row r="96" ht="46" customHeight="1">
       <c r="A96" s="7" t="inlineStr">
@@ -3969,11 +3975,11 @@
           <t>Several runs diverged in direct Steady mode due to reversed flow at the pressure outlet — a known failure mode for Newton-type steady solvers. Fix: run a short Transient burst (small dt, 50 timesteps, 50 max iterations/step) purely to let the flow settle direction, verify with 3 checks (zero reversed-flow messages / balanced mdot_in-mdot_out / flattened tau_wall), then switch Solver &gt; Time to Steady WITHOUT re-initializing and continue.</t>
         </is>
       </c>
-      <c r="B96" s="7" t="n"/>
-      <c r="C96" s="7" t="n"/>
-      <c r="D96" s="7" t="n"/>
-      <c r="E96" s="7" t="n"/>
-      <c r="F96" s="7" t="n"/>
+      <c r="B96" s="13" t="n"/>
+      <c r="C96" s="13" t="n"/>
+      <c r="D96" s="13" t="n"/>
+      <c r="E96" s="13" t="n"/>
+      <c r="F96" s="14" t="n"/>
     </row>
     <row r="98" ht="18" customHeight="1">
       <c r="A98" s="3" t="inlineStr">
@@ -3981,11 +3987,11 @@
           <t>What is proven vs. what is practitioner consensus — be precise about this if asked by advisor/committee</t>
         </is>
       </c>
-      <c r="B98" s="3" t="n"/>
-      <c r="C98" s="3" t="n"/>
-      <c r="D98" s="3" t="n"/>
-      <c r="E98" s="3" t="n"/>
-      <c r="F98" s="3" t="n"/>
+      <c r="B98" s="13" t="n"/>
+      <c r="C98" s="13" t="n"/>
+      <c r="D98" s="13" t="n"/>
+      <c r="E98" s="13" t="n"/>
+      <c r="F98" s="14" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="4" t="inlineStr">
@@ -4078,11 +4084,11 @@
           <t>Defensible framing for presentation: "This is an application of pseudo-transient continuation (Kelley &amp; Keyes, 1998), a peer-reviewed globalization method for stalled Newton-type steady solvers. We applied it only where the steady solver demonstrably failed (reversed flow at the outlet), verified recovery with three independent, measurable, documented criteria (surface report plots per the Fluent Tutorial Guide), and switched to Steady without re-initializing to preserve the fixed field. The specific Fluent implementation detail is supported by consistent field practitioner reports, not an ANSYS manual citation — stated honestly, not oversold."</t>
         </is>
       </c>
-      <c r="B105" s="23" t="n"/>
-      <c r="C105" s="23" t="n"/>
-      <c r="D105" s="23" t="n"/>
-      <c r="E105" s="23" t="n"/>
-      <c r="F105" s="23" t="n"/>
+      <c r="B105" s="13" t="n"/>
+      <c r="C105" s="13" t="n"/>
+      <c r="D105" s="13" t="n"/>
+      <c r="E105" s="13" t="n"/>
+      <c r="F105" s="14" t="n"/>
     </row>
     <row r="106" ht="30" customHeight="1">
       <c r="A106" s="7" t="inlineStr">
@@ -4090,11 +4096,88 @@
           <t>TODO before final thesis submission: pull the actual Kelley &amp; Keyes (1998) PDF and cite the specific page/section describing the small-to-large timestep growth strategy; if possible, also locate an official ANSYS Fluent Theory Guide or User Guide passage on pseudo-time-stepping / solution stabilization to strengthen the Fluent-specific link.</t>
         </is>
       </c>
-      <c r="B106" s="7" t="n"/>
-      <c r="C106" s="7" t="n"/>
-      <c r="D106" s="7" t="n"/>
-      <c r="E106" s="7" t="n"/>
-      <c r="F106" s="7" t="n"/>
+      <c r="B106" s="13" t="n"/>
+      <c r="C106" s="13" t="n"/>
+      <c r="D106" s="13" t="n"/>
+      <c r="E106" s="13" t="n"/>
+      <c r="F106" s="14" t="n"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="56" t="inlineStr">
+        <is>
+          <t>Methodology Note - Under-Relaxation (official, documented alternative to the transient-recovery fix above)</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="57" t="inlineStr">
+        <is>
+          <t>ANSYS Fluent's own User Guide states default under-relaxation factors (URFs) are tuned for the largest number of cases, but nonlinear/turbulent problems may need lower factors from the start, and recommends reducing them (in steps of about 0.1-0.2) specifically when residuals keep rising instead of settling in the first iterations - the same symptom seen in the diverging runs above. This is the officially documented first-line fix for steady-solver divergence, distinct from the transient-switch method.</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="56" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="57" t="inlineStr">
+        <is>
+          <t>Lowering URFs (momentum, pressure) is the standard, vendor-documented response to steady-state divergence/rising residuals.</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="57" t="inlineStr">
+        <is>
+          <t>Reducing the pressure-outlet backflow instability can also be addressed via boundary placement/setup (outlet sited further downstream in uniform flow, correct backflow turbulence/temperature values) rather than solver settings alone - a root-cause angle distinct from both under-relaxation and transient-switching.</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="56" t="inlineStr">
+        <is>
+          <t>Status: not yet applied to any of the recovered runs (39, 47, 52, 54, Stage-4 re-runs) - those were fixed via the transient method above before this alternative was identified. Recommend citing under-relaxation as the officially-backed method if the committee or advisor specifically objects to the transient-switch, since it carries a vendor-documentation citation the transient method lacks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="56" t="inlineStr">
+        <is>
+          <t>References</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="57" t="inlineStr">
+        <is>
+          <t>ANSYS Fluent User's Guide, Under-Relaxation of Variables (ENEA mirror) - https://wwwafs.portici.enea.it/project/neptunius/docs/fluent/html/ug/node786.htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="57" t="inlineStr">
+        <is>
+          <t>ANSYS Innovation Space forum, 'Under-Relaxation Factors' - https://innovationspace.ansys.com/forum/forums/topic/under-relaxation-factors-4</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="57" t="inlineStr">
+        <is>
+          <t>CFD Online forum, 'Reverse flow pressure outlet' - https://cfd-online.com/Forums/fluent/94824-reverse-flow-pressure-outlet.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="57" t="inlineStr">
+        <is>
+          <t>ANSYS Innovation Space forum, pseudo-transient relaxation vs. outflow condition on a backflow case - https://innovationspace.ansys.com/forum/?p=247383</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="44">

</xml_diff>